<commit_message>
Dodana tablica Adresy do bazy, dodany Kraj do csv, lepiej działa fuzzy from left to right.
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17FF032-C91D-458E-A7C5-8D1952984883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{900D4DC6-B755-4B15-9600-676C5D43586D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B40A3022-A911-427C-BBA3-985EEBB0CEC6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="43">
   <si>
     <t>KEN</t>
   </si>
@@ -159,6 +159,12 @@
   </si>
   <si>
     <t>Bielsko-Biała</t>
+  </si>
+  <si>
+    <t>II Pułku Lotniczego</t>
+  </si>
+  <si>
+    <t>2 Pułku Lotniczego</t>
   </si>
 </sst>
 </file>
@@ -531,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83832BEB-642D-4FE8-AB82-A805522C5706}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.28515625" customWidth="1"/>
@@ -758,6 +764,17 @@
         <v>40</v>
       </c>
     </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
poprawki do korekt nazw ulic
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -1,23 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664FD3CC-FD5B-435C-A24E-6533022F876E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4507"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B40A3022-A911-427C-BBA3-985EEBB0CEC6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="23256" windowHeight="13176"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="125725"/>
+  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="70">
   <si>
     <t>KEN</t>
   </si>
@@ -243,12 +237,6 @@
   </si>
   <si>
     <t>.Lecia</t>
-  </si>
-  <si>
-    <t>0.-</t>
-  </si>
-  <si>
-    <t>0-</t>
   </si>
   <si>
     <t>*-</t>
@@ -257,8 +245,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -351,7 +339,7 @@
     </a:clrScheme>
     <a:fontScheme name="Pakiet Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -403,7 +391,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -617,22 +605,22 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83832BEB-642D-4FE8-AB82-A805522C5706}">
-  <dimension ref="A1:C40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C39"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="2" max="2" width="29.28515625" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.296875" customWidth="1"/>
+    <col min="3" max="3" width="37.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -643,7 +631,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -654,7 +642,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -665,7 +653,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -676,7 +664,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -687,7 +675,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -698,7 +686,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -709,7 +697,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -720,7 +708,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -731,7 +719,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -742,7 +730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -753,7 +741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -764,7 +752,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -775,7 +763,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -786,7 +774,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -797,7 +785,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -808,7 +796,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -819,7 +807,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -830,7 +818,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -841,7 +829,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -852,7 +840,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -863,7 +851,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -874,7 +862,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -885,15 +873,18 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>10</v>
+      </c>
       <c r="B24" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C24" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>10</v>
       </c>
@@ -904,173 +895,162 @@
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3">
       <c r="A26" t="s">
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>69</v>
-      </c>
-      <c r="C26" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" t="s">
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3">
       <c r="A28" t="s">
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>67</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="C28" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C29" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3">
       <c r="A30" t="s">
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C30" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
       <c r="A31" t="s">
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="C31" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3">
       <c r="A32" t="s">
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C32" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
       <c r="A33" t="s">
         <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C33" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
       <c r="A34" t="s">
         <v>10</v>
       </c>
       <c r="B34" t="s">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="C34" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3">
       <c r="A35" t="s">
         <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C35" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
       <c r="A36" t="s">
         <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C36" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
       <c r="A37" t="s">
         <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="C37" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
       <c r="A38" t="s">
         <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C38" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
       <c r="A39" t="s">
         <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C39" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>10</v>
-      </c>
-      <c r="B40" t="s">
-        <v>47</v>
-      </c>
-      <c r="C40" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C40">
+  <sortState ref="A2:C40">
     <sortCondition ref="A2:A40"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Walka z prefiksami ksiądz i generał.
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -1,36 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4507"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91984DA7-286D-46FB-B53E-CE82E095EEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="23256" windowHeight="13176"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="125725"/>
-  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="92">
   <si>
     <t>KEN</t>
   </si>
@@ -240,13 +235,79 @@
   </si>
   <si>
     <t>*-</t>
+  </si>
+  <si>
+    <t>Gorzów Wlkp.</t>
+  </si>
+  <si>
+    <t>Gorzów Wielkopolski</t>
+  </si>
+  <si>
+    <t>Bystra Śląska</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bystra </t>
+  </si>
+  <si>
+    <t>Grodzisk Wlkp.</t>
+  </si>
+  <si>
+    <t>Grodzisk Wielkopolski</t>
+  </si>
+  <si>
+    <t>Piotrków Tryb.</t>
+  </si>
+  <si>
+    <t>Piotrków Trybunalski</t>
+  </si>
+  <si>
+    <t>Ruda Śl.</t>
+  </si>
+  <si>
+    <t>Ruda Śląska</t>
+  </si>
+  <si>
+    <t>Sędziszów Młp.</t>
+  </si>
+  <si>
+    <t>Sędziszów Małopolski</t>
+  </si>
+  <si>
+    <t>Siemianowice Śl.</t>
+  </si>
+  <si>
+    <t>Siemianowice Śląskie</t>
+  </si>
+  <si>
+    <t>Sokołów Młp.</t>
+  </si>
+  <si>
+    <t>Sokołów Małopolski</t>
+  </si>
+  <si>
+    <t>Stargard Szczeciński</t>
+  </si>
+  <si>
+    <t>Stargard</t>
+  </si>
+  <si>
+    <t>Tomaszów Maz.</t>
+  </si>
+  <si>
+    <t>Tomaszów Mazowiecki</t>
+  </si>
+  <si>
+    <t>Wodzisław Śl.</t>
+  </si>
+  <si>
+    <t>Wodzisław Śląski</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -605,22 +666,22 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.296875" customWidth="1"/>
-    <col min="3" max="3" width="37.3984375" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -631,7 +692,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -642,7 +703,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -653,7 +714,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -664,7 +725,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -675,7 +736,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -686,7 +747,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -697,361 +758,493 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
       <c r="B8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22" t="s">
         <v>0</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C22" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" t="s">
         <v>4</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C23" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" t="s">
         <v>5</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C24" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" t="s">
         <v>15</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C25" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" t="s">
         <v>24</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C26" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>10</v>
+      </c>
+      <c r="B27" t="s">
         <v>26</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C27" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" t="s">
         <v>2</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C28" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>10</v>
+      </c>
+      <c r="B29" t="s">
         <v>16</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C29" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>10</v>
+      </c>
+      <c r="B30" t="s">
         <v>18</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C30" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B19" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>10</v>
+      </c>
+      <c r="B31" t="s">
         <v>20</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
-        <v>10</v>
-      </c>
-      <c r="B20" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B32" t="s">
         <v>23</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C32" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
-      <c r="A21" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
         <v>41</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C33" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
-        <v>10</v>
-      </c>
-      <c r="B22" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" t="s">
         <v>43</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C34" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
-      <c r="A23" t="s">
-        <v>10</v>
-      </c>
-      <c r="B23" s="1" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C35" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
-      <c r="A24" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24" s="1" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C36" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
-      <c r="A25" t="s">
-        <v>10</v>
-      </c>
-      <c r="B25" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>10</v>
+      </c>
+      <c r="B37" t="s">
         <v>68</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C37" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
-      <c r="A26" t="s">
-        <v>10</v>
-      </c>
-      <c r="B26" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38" t="s">
         <v>53</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C38" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
-        <v>10</v>
-      </c>
-      <c r="B27" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>10</v>
+      </c>
+      <c r="B39" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C39" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
-      <c r="A28" t="s">
-        <v>10</v>
-      </c>
-      <c r="B28" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>10</v>
+      </c>
+      <c r="B40" t="s">
         <v>55</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C40" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
-      <c r="A29" t="s">
-        <v>10</v>
-      </c>
-      <c r="B29" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>10</v>
+      </c>
+      <c r="B41" t="s">
         <v>59</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C41" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>10</v>
-      </c>
-      <c r="B30" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>10</v>
+      </c>
+      <c r="B42" t="s">
         <v>57</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C42" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
-      <c r="A31" t="s">
-        <v>10</v>
-      </c>
-      <c r="B31" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>10</v>
+      </c>
+      <c r="B43" t="s">
         <v>25</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C43" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
-      <c r="A32" t="s">
-        <v>10</v>
-      </c>
-      <c r="B32" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>10</v>
+      </c>
+      <c r="B44" t="s">
         <v>27</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C44" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
-      <c r="A33" t="s">
-        <v>10</v>
-      </c>
-      <c r="B33" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>10</v>
+      </c>
+      <c r="B45" t="s">
         <v>14</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C45" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>10</v>
-      </c>
-      <c r="B34" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>10</v>
+      </c>
+      <c r="B46" t="s">
         <v>66</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C46" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
-      <c r="A35" t="s">
-        <v>10</v>
-      </c>
-      <c r="B35" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>10</v>
+      </c>
+      <c r="B47" t="s">
         <v>61</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C47" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>10</v>
-      </c>
-      <c r="B36" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>10</v>
+      </c>
+      <c r="B48" t="s">
         <v>63</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C48" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>10</v>
-      </c>
-      <c r="B37" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>10</v>
+      </c>
+      <c r="B49" t="s">
         <v>49</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C49" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
-      <c r="A38" t="s">
-        <v>10</v>
-      </c>
-      <c r="B38" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>10</v>
+      </c>
+      <c r="B50" t="s">
         <v>45</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C50" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>10</v>
-      </c>
-      <c r="B39" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>10</v>
+      </c>
+      <c r="B51" t="s">
         <v>47</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C51" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:C40">
-    <sortCondition ref="A2:A40"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C52">
+    <sortCondition ref="A2:A52"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Połączone ładowanie CechUlic, bo było w 2 miejscach
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -1,23 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4507"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91984DA7-286D-46FB-B53E-CE82E095EEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23256" windowHeight="13176"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="125725"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="98">
   <si>
     <t>KEN</t>
   </si>
@@ -168,12 +162,6 @@
     <t>Chopina</t>
   </si>
   <si>
-    <t>Curie-Skłodowskiej</t>
-  </si>
-  <si>
-    <t>Skłodowskiej-Curie</t>
-  </si>
-  <si>
     <t>Tysiąclecia</t>
   </si>
   <si>
@@ -301,13 +289,37 @@
   </si>
   <si>
     <t>Wodzisław Śląski</t>
+  </si>
+  <si>
+    <t>ZHP</t>
+  </si>
+  <si>
+    <t>Związku Harcerstwa Polskiego</t>
+  </si>
+  <si>
+    <t>PTTK</t>
+  </si>
+  <si>
+    <t>Polskiego Towarzystwa Turystyczno-Krajoznawczego</t>
+  </si>
+  <si>
+    <t>Św. Św.</t>
+  </si>
+  <si>
+    <t>Świętych</t>
+  </si>
+  <si>
+    <t>*AK*</t>
+  </si>
+  <si>
+    <t>*Armii Krajowej*</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -666,22 +678,22 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C54"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="2" max="2" width="29.28515625" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.296875" customWidth="1"/>
+    <col min="3" max="3" width="37.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -692,7 +704,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -703,7 +715,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -714,7 +726,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -725,7 +737,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -736,7 +748,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -747,7 +759,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -758,18 +770,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -780,7 +792,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -791,40 +803,40 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
       <c r="B11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>70</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
         <v>72</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C13" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C13" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -835,84 +847,84 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>11</v>
       </c>
       <c r="B15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
         <v>82</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" t="s">
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" t="s">
         <v>84</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C18" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" t="s">
-        <v>80</v>
-      </c>
-      <c r="C17" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>11</v>
-      </c>
-      <c r="B18" t="s">
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
         <v>86</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>11</v>
-      </c>
-      <c r="B19" t="s">
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" t="s">
         <v>88</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C20" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>11</v>
-      </c>
-      <c r="B20" t="s">
-        <v>90</v>
-      </c>
-      <c r="C20" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C21" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -923,7 +935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -934,7 +946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -945,7 +957,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>10</v>
       </c>
@@ -956,7 +968,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3">
       <c r="A26" t="s">
         <v>10</v>
       </c>
@@ -967,7 +979,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -978,7 +990,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3">
       <c r="A28" t="s">
         <v>10</v>
       </c>
@@ -989,7 +1001,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>10</v>
       </c>
@@ -1000,7 +1012,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3">
       <c r="A30" t="s">
         <v>10</v>
       </c>
@@ -1011,7 +1023,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3">
       <c r="A31" t="s">
         <v>10</v>
       </c>
@@ -1022,7 +1034,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3">
       <c r="A32" t="s">
         <v>10</v>
       </c>
@@ -1033,7 +1045,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3">
       <c r="A33" t="s">
         <v>10</v>
       </c>
@@ -1044,7 +1056,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3">
       <c r="A34" t="s">
         <v>10</v>
       </c>
@@ -1055,95 +1067,95 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3">
       <c r="A35" t="s">
         <v>10</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C35" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>10</v>
+      </c>
+      <c r="B37" t="s">
+        <v>66</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C35" t="s">
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>10</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C36" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>10</v>
-      </c>
-      <c r="B37" t="s">
-        <v>68</v>
-      </c>
-      <c r="C37" s="1" t="s">
+      <c r="C38" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>10</v>
+      </c>
+      <c r="B39" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>10</v>
+      </c>
+      <c r="B40" t="s">
+        <v>53</v>
+      </c>
+      <c r="C40" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>10</v>
-      </c>
-      <c r="B38" t="s">
-        <v>53</v>
-      </c>
-      <c r="C38" s="1" t="s">
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>10</v>
+      </c>
+      <c r="B41" t="s">
+        <v>57</v>
+      </c>
+      <c r="C41" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>10</v>
-      </c>
-      <c r="B39" t="s">
-        <v>67</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>10</v>
-      </c>
-      <c r="B40" t="s">
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>10</v>
+      </c>
+      <c r="B42" t="s">
         <v>55</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C42" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>10</v>
-      </c>
-      <c r="B41" t="s">
-        <v>59</v>
-      </c>
-      <c r="C41" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>10</v>
-      </c>
-      <c r="B42" t="s">
-        <v>57</v>
-      </c>
-      <c r="C42" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3">
       <c r="A43" t="s">
         <v>10</v>
       </c>
@@ -1151,10 +1163,10 @@
         <v>25</v>
       </c>
       <c r="C43" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
       <c r="A44" t="s">
         <v>10</v>
       </c>
@@ -1162,10 +1174,10 @@
         <v>27</v>
       </c>
       <c r="C44" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
       <c r="A45" t="s">
         <v>10</v>
       </c>
@@ -1173,54 +1185,54 @@
         <v>14</v>
       </c>
       <c r="C45" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
       <c r="A46" t="s">
         <v>10</v>
       </c>
       <c r="B46" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C46" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
       <c r="A47" t="s">
         <v>10</v>
       </c>
       <c r="B47" t="s">
+        <v>59</v>
+      </c>
+      <c r="C47" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>10</v>
+      </c>
+      <c r="B48" t="s">
         <v>61</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>10</v>
-      </c>
-      <c r="B48" t="s">
-        <v>63</v>
-      </c>
-      <c r="C48" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3">
       <c r="A49" t="s">
         <v>10</v>
       </c>
       <c r="B49" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C49" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
       <c r="A50" t="s">
         <v>10</v>
       </c>
@@ -1231,19 +1243,52 @@
         <v>46</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3">
       <c r="A51" t="s">
         <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="C51" t="s">
-        <v>48</v>
+        <v>91</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
+        <v>10</v>
+      </c>
+      <c r="B52" t="s">
+        <v>96</v>
+      </c>
+      <c r="C52" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>10</v>
+      </c>
+      <c r="B53" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>10</v>
+      </c>
+      <c r="B54" t="s">
+        <v>94</v>
+      </c>
+      <c r="C54" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C52">
+  <sortState ref="A2:C52">
     <sortCondition ref="A2:A52"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fajnie wszystko działa, 200 błędów ładowania kodów pocztowych
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -1,17 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4507"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D57580C-4B15-4EB0-964C-9DA2C5BFB78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23256" windowHeight="13176"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="125725"/>
-  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -19,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="149">
   <si>
     <t>KEN</t>
   </si>
@@ -171,12 +177,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>-*</t>
-  </si>
-  <si>
-    <t>*lecia</t>
-  </si>
-  <si>
     <t>-lecia</t>
   </si>
   <si>
@@ -216,15 +216,6 @@
     <t>Trzydziestolecia</t>
   </si>
   <si>
-    <t>*Lecia</t>
-  </si>
-  <si>
-    <t>.Lecia</t>
-  </si>
-  <si>
-    <t>*-</t>
-  </si>
-  <si>
     <t>Gorzów Wlkp.</t>
   </si>
   <si>
@@ -309,17 +300,185 @@
     <t>Świętych</t>
   </si>
   <si>
-    <t>*AK*</t>
-  </si>
-  <si>
-    <t>*Armii Krajowej*</t>
+    <t>AK</t>
+  </si>
+  <si>
+    <t>!-*</t>
+  </si>
+  <si>
+    <t>!*-</t>
+  </si>
+  <si>
+    <t>!.Lecia</t>
+  </si>
+  <si>
+    <t>!*lecia</t>
+  </si>
+  <si>
+    <t>!*Lecia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">!*van* </t>
+  </si>
+  <si>
+    <t>*van_</t>
+  </si>
+  <si>
+    <t xml:space="preserve">!*de* </t>
+  </si>
+  <si>
+    <t>*de_</t>
+  </si>
+  <si>
+    <t>!*la*</t>
+  </si>
+  <si>
+    <t>*la_</t>
+  </si>
+  <si>
+    <t>0 Roku</t>
+  </si>
+  <si>
+    <t>1 Roku</t>
+  </si>
+  <si>
+    <t>2 Roku</t>
+  </si>
+  <si>
+    <t>3 Roku</t>
+  </si>
+  <si>
+    <t>4 Roku</t>
+  </si>
+  <si>
+    <t>5 Roku</t>
+  </si>
+  <si>
+    <t>6 Roku</t>
+  </si>
+  <si>
+    <t>7 Roku</t>
+  </si>
+  <si>
+    <t>8 Roku</t>
+  </si>
+  <si>
+    <t>9 Roku</t>
+  </si>
+  <si>
+    <t>!0 r.</t>
+  </si>
+  <si>
+    <t>!1 r.</t>
+  </si>
+  <si>
+    <t>!2 r.</t>
+  </si>
+  <si>
+    <t>!3 r.</t>
+  </si>
+  <si>
+    <t>!4 r.</t>
+  </si>
+  <si>
+    <t>!5 r.</t>
+  </si>
+  <si>
+    <t>!6 r.</t>
+  </si>
+  <si>
+    <t>!7 r.</t>
+  </si>
+  <si>
+    <t>!8 r.</t>
+  </si>
+  <si>
+    <t>!9 r.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">!*von* </t>
+  </si>
+  <si>
+    <t>*von_</t>
+  </si>
+  <si>
+    <t xml:space="preserve">!*da* </t>
+  </si>
+  <si>
+    <t>*da_</t>
+  </si>
+  <si>
+    <t>Dzierżonia</t>
+  </si>
+  <si>
+    <t>Dzierżona</t>
+  </si>
+  <si>
+    <t>imienia</t>
+  </si>
+  <si>
+    <t>im.</t>
+  </si>
+  <si>
+    <t>Kolbe</t>
+  </si>
+  <si>
+    <t>Kolbego</t>
+  </si>
+  <si>
+    <t>!*z*</t>
+  </si>
+  <si>
+    <t>*z_</t>
+  </si>
+  <si>
+    <t>!*ze*</t>
+  </si>
+  <si>
+    <t>*ze_</t>
+  </si>
+  <si>
+    <t>!*le*</t>
+  </si>
+  <si>
+    <t>*le_</t>
+  </si>
+  <si>
+    <t>Ułanów Wlkp.</t>
+  </si>
+  <si>
+    <t>Ułanów Wielkopolskich</t>
+  </si>
+  <si>
+    <t>Piechoty Wlkp.</t>
+  </si>
+  <si>
+    <t>Piechoty Wielkopolskiej</t>
+  </si>
+  <si>
+    <t>Ducha Świętego</t>
+  </si>
+  <si>
+    <t>świętego Ducha</t>
+  </si>
+  <si>
+    <t>Maryi</t>
+  </si>
+  <si>
+    <t>Marii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">!*del* </t>
+  </si>
+  <si>
+    <t>*del_</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -678,22 +837,22 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C80"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.296875" customWidth="1"/>
-    <col min="3" max="3" width="37.3984375" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -704,7 +863,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -715,7 +874,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -726,7 +885,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -737,7 +896,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -748,7 +907,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -759,7 +918,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -770,18 +929,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -792,7 +951,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -803,40 +962,40 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
       <c r="B11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" t="s">
         <v>68</v>
       </c>
-      <c r="C11" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>70</v>
-      </c>
-      <c r="C12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -847,84 +1006,84 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
       <c r="B15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18" t="s">
         <v>80</v>
       </c>
-      <c r="C15" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="C19" t="s">
         <v>82</v>
       </c>
-      <c r="C16" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" t="s">
-        <v>78</v>
-      </c>
-      <c r="C17" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>11</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="C20" t="s">
         <v>84</v>
       </c>
-      <c r="C18" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>11</v>
-      </c>
-      <c r="B19" t="s">
-        <v>86</v>
-      </c>
-      <c r="C19" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
-        <v>11</v>
-      </c>
-      <c r="B20" t="s">
-        <v>88</v>
-      </c>
-      <c r="C20" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C21" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -935,7 +1094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -946,7 +1105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -957,7 +1116,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>10</v>
       </c>
@@ -968,7 +1127,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>10</v>
       </c>
@@ -979,7 +1138,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -990,7 +1149,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>10</v>
       </c>
@@ -1001,7 +1160,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>10</v>
       </c>
@@ -1012,7 +1171,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>10</v>
       </c>
@@ -1023,273 +1182,559 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>10</v>
       </c>
       <c r="B31" t="s">
+        <v>141</v>
+      </c>
+      <c r="C31" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B32" t="s">
+        <v>139</v>
+      </c>
+      <c r="C32" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
         <v>20</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
-      <c r="A32" t="s">
-        <v>10</v>
-      </c>
-      <c r="B32" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" t="s">
         <v>23</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C34" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
-      <c r="A33" t="s">
-        <v>10</v>
-      </c>
-      <c r="B33" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" t="s">
         <v>41</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C35" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>10</v>
-      </c>
-      <c r="B34" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" t="s">
         <v>43</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C36" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
-      <c r="A35" t="s">
-        <v>10</v>
-      </c>
-      <c r="B35" s="1" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>10</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C37" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C38" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>10</v>
+      </c>
+      <c r="B39" t="s">
+        <v>94</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C35" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>10</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C36" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>10</v>
-      </c>
-      <c r="B37" t="s">
-        <v>66</v>
-      </c>
-      <c r="C37" s="1" t="s">
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>10</v>
+      </c>
+      <c r="B40" t="s">
+        <v>95</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>10</v>
+      </c>
+      <c r="B41" t="s">
+        <v>96</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>10</v>
+      </c>
+      <c r="B42" t="s">
+        <v>51</v>
+      </c>
+      <c r="C42" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
-      <c r="A38" t="s">
-        <v>10</v>
-      </c>
-      <c r="B38" t="s">
-        <v>51</v>
-      </c>
-      <c r="C38" s="1" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>10</v>
+      </c>
+      <c r="B43" t="s">
+        <v>55</v>
+      </c>
+      <c r="C43" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>10</v>
-      </c>
-      <c r="B39" t="s">
-        <v>65</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" t="s">
-        <v>10</v>
-      </c>
-      <c r="B40" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>10</v>
+      </c>
+      <c r="B44" t="s">
         <v>53</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C44" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
-      <c r="A41" t="s">
-        <v>10</v>
-      </c>
-      <c r="B41" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>10</v>
+      </c>
+      <c r="B45" t="s">
+        <v>25</v>
+      </c>
+      <c r="C45" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>10</v>
+      </c>
+      <c r="B46" t="s">
+        <v>27</v>
+      </c>
+      <c r="C46" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>10</v>
+      </c>
+      <c r="B47" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>10</v>
+      </c>
+      <c r="B48" t="s">
+        <v>62</v>
+      </c>
+      <c r="C48" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>10</v>
+      </c>
+      <c r="B49" t="s">
         <v>57</v>
       </c>
-      <c r="C41" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" t="s">
-        <v>10</v>
-      </c>
-      <c r="B42" t="s">
-        <v>55</v>
-      </c>
-      <c r="C42" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" t="s">
-        <v>10</v>
-      </c>
-      <c r="B43" t="s">
-        <v>25</v>
-      </c>
-      <c r="C43" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>10</v>
-      </c>
-      <c r="B44" t="s">
-        <v>27</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="C49" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
-      <c r="A45" t="s">
-        <v>10</v>
-      </c>
-      <c r="B45" t="s">
-        <v>14</v>
-      </c>
-      <c r="C45" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" t="s">
-        <v>10</v>
-      </c>
-      <c r="B46" t="s">
-        <v>64</v>
-      </c>
-      <c r="C46" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" t="s">
-        <v>10</v>
-      </c>
-      <c r="B47" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>10</v>
+      </c>
+      <c r="B50" t="s">
         <v>59</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C50" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
-      <c r="A48" t="s">
-        <v>10</v>
-      </c>
-      <c r="B48" t="s">
-        <v>61</v>
-      </c>
-      <c r="C48" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" t="s">
-        <v>10</v>
-      </c>
-      <c r="B49" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>10</v>
+      </c>
+      <c r="B51" t="s">
         <v>47</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C51" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
-      <c r="A50" t="s">
-        <v>10</v>
-      </c>
-      <c r="B50" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>10</v>
+      </c>
+      <c r="B52" t="s">
         <v>45</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C52" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
-      <c r="A51" t="s">
-        <v>10</v>
-      </c>
-      <c r="B51" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>10</v>
+      </c>
+      <c r="B53" t="s">
+        <v>85</v>
+      </c>
+      <c r="C53" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>10</v>
+      </c>
+      <c r="B54" t="s">
+        <v>91</v>
+      </c>
+      <c r="C54" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>10</v>
+      </c>
+      <c r="B55" t="s">
+        <v>87</v>
+      </c>
+      <c r="C55" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>10</v>
+      </c>
+      <c r="B56" t="s">
+        <v>89</v>
+      </c>
+      <c r="C56" t="s">
         <v>90</v>
       </c>
-      <c r="C51" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" t="s">
-        <v>10</v>
-      </c>
-      <c r="B52" t="s">
-        <v>96</v>
-      </c>
-      <c r="C52" t="s">
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>10</v>
+      </c>
+      <c r="B57" t="s">
+        <v>123</v>
+      </c>
+      <c r="C57" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>10</v>
+      </c>
+      <c r="B58" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" t="s">
-        <v>10</v>
-      </c>
-      <c r="B53" t="s">
-        <v>92</v>
-      </c>
-      <c r="C53" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54" t="s">
-        <v>10</v>
-      </c>
-      <c r="B54" t="s">
-        <v>94</v>
-      </c>
-      <c r="C54" t="s">
-        <v>95</v>
+      <c r="C58" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>10</v>
+      </c>
+      <c r="B59" t="s">
+        <v>99</v>
+      </c>
+      <c r="C59" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>10</v>
+      </c>
+      <c r="B60" t="s">
+        <v>125</v>
+      </c>
+      <c r="C60" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>10</v>
+      </c>
+      <c r="B61" t="s">
+        <v>137</v>
+      </c>
+      <c r="C61" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>10</v>
+      </c>
+      <c r="B62" t="s">
+        <v>147</v>
+      </c>
+      <c r="C62" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>10</v>
+      </c>
+      <c r="B63" t="s">
+        <v>101</v>
+      </c>
+      <c r="C63" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>10</v>
+      </c>
+      <c r="B64" t="s">
+        <v>113</v>
+      </c>
+      <c r="C64" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>10</v>
+      </c>
+      <c r="B65" t="s">
+        <v>114</v>
+      </c>
+      <c r="C65" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>10</v>
+      </c>
+      <c r="B66" t="s">
+        <v>115</v>
+      </c>
+      <c r="C66" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>10</v>
+      </c>
+      <c r="B67" t="s">
+        <v>116</v>
+      </c>
+      <c r="C67" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>10</v>
+      </c>
+      <c r="B68" t="s">
+        <v>117</v>
+      </c>
+      <c r="C68" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>10</v>
+      </c>
+      <c r="B69" t="s">
+        <v>118</v>
+      </c>
+      <c r="C69" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>10</v>
+      </c>
+      <c r="B70" t="s">
+        <v>119</v>
+      </c>
+      <c r="C70" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>10</v>
+      </c>
+      <c r="B71" t="s">
+        <v>120</v>
+      </c>
+      <c r="C71" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>10</v>
+      </c>
+      <c r="B72" t="s">
+        <v>121</v>
+      </c>
+      <c r="C72" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>10</v>
+      </c>
+      <c r="B73" t="s">
+        <v>122</v>
+      </c>
+      <c r="C73" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>10</v>
+      </c>
+      <c r="B74" t="s">
+        <v>133</v>
+      </c>
+      <c r="C74" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>10</v>
+      </c>
+      <c r="B75" t="s">
+        <v>135</v>
+      </c>
+      <c r="C75" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>10</v>
+      </c>
+      <c r="B76" t="s">
+        <v>127</v>
+      </c>
+      <c r="C76" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>10</v>
+      </c>
+      <c r="B77" t="s">
+        <v>129</v>
+      </c>
+      <c r="C77" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>10</v>
+      </c>
+      <c r="B78" t="s">
+        <v>131</v>
+      </c>
+      <c r="C78" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>10</v>
+      </c>
+      <c r="B79" t="s">
+        <v>143</v>
+      </c>
+      <c r="C79" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>10</v>
+      </c>
+      <c r="B80" t="s">
+        <v>145</v>
+      </c>
+      <c r="C80" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:C52">
-    <sortCondition ref="A2:A52"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C54">
+    <sortCondition ref="A2:A54"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Kody pocztowe udrożnione, Zostało jeszcze około 240 niezgodności
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D57580C-4B15-4EB0-964C-9DA2C5BFB78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A71BC41-CECD-4906-99FF-709B48AB41B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="171">
   <si>
     <t>KEN</t>
   </si>
@@ -472,6 +472,72 @@
   </si>
   <si>
     <t>*del_</t>
+  </si>
+  <si>
+    <t>Dowbor-</t>
+  </si>
+  <si>
+    <t>Dowbora-</t>
+  </si>
+  <si>
+    <t>P.por.</t>
+  </si>
+  <si>
+    <t>podporucznik</t>
+  </si>
+  <si>
+    <t>bpa</t>
+  </si>
+  <si>
+    <t>Francesco</t>
+  </si>
+  <si>
+    <t>Francesca</t>
+  </si>
+  <si>
+    <t>Nullo</t>
+  </si>
+  <si>
+    <t>Nulla</t>
+  </si>
+  <si>
+    <t>Hauke-</t>
+  </si>
+  <si>
+    <t>Haukego-</t>
+  </si>
+  <si>
+    <t>doktora</t>
+  </si>
+  <si>
+    <t>dra</t>
+  </si>
+  <si>
+    <t>biskupa</t>
+  </si>
+  <si>
+    <t>Josepha Conrada</t>
+  </si>
+  <si>
+    <t>Józefa Korzeniowskiego</t>
+  </si>
+  <si>
+    <t>RP</t>
+  </si>
+  <si>
+    <t>Rzeczpospolitej Polskiej</t>
+  </si>
+  <si>
+    <t>NSZZ</t>
+  </si>
+  <si>
+    <t>Niezależnego Samodzielnego Związku Zawodowego</t>
+  </si>
+  <si>
+    <t>Bacewiczówny</t>
+  </si>
+  <si>
+    <t>Bacewicz</t>
   </si>
 </sst>
 </file>
@@ -845,7 +911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.28515625" customWidth="1"/>
@@ -1732,6 +1798,127 @@
         <v>146</v>
       </c>
     </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>10</v>
+      </c>
+      <c r="B81" t="s">
+        <v>149</v>
+      </c>
+      <c r="C81" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>10</v>
+      </c>
+      <c r="B82" t="s">
+        <v>151</v>
+      </c>
+      <c r="C82" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>10</v>
+      </c>
+      <c r="B83" t="s">
+        <v>153</v>
+      </c>
+      <c r="C83" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>10</v>
+      </c>
+      <c r="B84" t="s">
+        <v>161</v>
+      </c>
+      <c r="C84" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>10</v>
+      </c>
+      <c r="B85" t="s">
+        <v>154</v>
+      </c>
+      <c r="C85" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>10</v>
+      </c>
+      <c r="B86" t="s">
+        <v>156</v>
+      </c>
+      <c r="C86" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>10</v>
+      </c>
+      <c r="B87" t="s">
+        <v>158</v>
+      </c>
+      <c r="C87" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>10</v>
+      </c>
+      <c r="B88" t="s">
+        <v>163</v>
+      </c>
+      <c r="C88" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>10</v>
+      </c>
+      <c r="B89" t="s">
+        <v>165</v>
+      </c>
+      <c r="C89" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>10</v>
+      </c>
+      <c r="B90" t="s">
+        <v>167</v>
+      </c>
+      <c r="C90" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>10</v>
+      </c>
+      <c r="B91" t="s">
+        <v>169</v>
+      </c>
+      <c r="C91" t="s">
+        <v>170</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Działa, ładują się wszystkie Urzędy Skarbowe
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A71BC41-CECD-4906-99FF-709B48AB41B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B398410F-E4FC-4CC8-B132-F28FF3A22816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="173">
   <si>
     <t>KEN</t>
   </si>
@@ -538,6 +538,12 @@
   </si>
   <si>
     <t>Bacewicz</t>
+  </si>
+  <si>
+    <t>Boh. Warszawy</t>
+  </si>
+  <si>
+    <t>Bohaterów Warszawy</t>
   </si>
 </sst>
 </file>
@@ -911,7 +917,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.28515625" customWidth="1"/>
@@ -1297,10 +1303,10 @@
         <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>41</v>
+        <v>171</v>
       </c>
       <c r="C35" t="s">
-        <v>42</v>
+        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1308,21 +1314,21 @@
         <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>10</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>92</v>
+      <c r="B37" t="s">
+        <v>43</v>
       </c>
       <c r="C37" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1330,7 +1336,7 @@
         <v>10</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C38" t="s">
         <v>49</v>
@@ -1340,11 +1346,11 @@
       <c r="A39" t="s">
         <v>10</v>
       </c>
-      <c r="B39" t="s">
-        <v>94</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>50</v>
+      <c r="B39" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C39" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1352,7 +1358,7 @@
         <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>50</v>
@@ -1363,7 +1369,7 @@
         <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>50</v>
@@ -1374,10 +1380,10 @@
         <v>10</v>
       </c>
       <c r="B42" t="s">
-        <v>51</v>
-      </c>
-      <c r="C42" t="s">
-        <v>52</v>
+        <v>96</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1385,7 +1391,7 @@
         <v>10</v>
       </c>
       <c r="B43" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C43" t="s">
         <v>52</v>
@@ -1396,10 +1402,10 @@
         <v>10</v>
       </c>
       <c r="B44" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C44" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1407,7 +1413,7 @@
         <v>10</v>
       </c>
       <c r="B45" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="C45" t="s">
         <v>54</v>
@@ -1418,10 +1424,10 @@
         <v>10</v>
       </c>
       <c r="B46" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C46" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1429,10 +1435,10 @@
         <v>10</v>
       </c>
       <c r="B47" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="C47" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1440,7 +1446,7 @@
         <v>10</v>
       </c>
       <c r="B48" t="s">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="C48" t="s">
         <v>61</v>
@@ -1451,10 +1457,10 @@
         <v>10</v>
       </c>
       <c r="B49" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C49" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1462,10 +1468,10 @@
         <v>10</v>
       </c>
       <c r="B50" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C50" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1473,10 +1479,10 @@
         <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C51" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1484,10 +1490,10 @@
         <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C52" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1495,10 +1501,10 @@
         <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="C53" t="s">
-        <v>86</v>
+        <v>46</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1506,10 +1512,10 @@
         <v>10</v>
       </c>
       <c r="B54" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C54" t="s">
-        <v>22</v>
+        <v>86</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -1517,10 +1523,10 @@
         <v>10</v>
       </c>
       <c r="B55" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C55" t="s">
-        <v>88</v>
+        <v>22</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -1528,10 +1534,10 @@
         <v>10</v>
       </c>
       <c r="B56" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C56" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -1539,10 +1545,10 @@
         <v>10</v>
       </c>
       <c r="B57" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="C57" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -1550,10 +1556,10 @@
         <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="C58" t="s">
-        <v>98</v>
+        <v>124</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -1561,10 +1567,10 @@
         <v>10</v>
       </c>
       <c r="B59" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C59" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -1572,10 +1578,10 @@
         <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="C60" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -1583,10 +1589,10 @@
         <v>10</v>
       </c>
       <c r="B61" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C61" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -1594,10 +1600,10 @@
         <v>10</v>
       </c>
       <c r="B62" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C62" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -1605,10 +1611,10 @@
         <v>10</v>
       </c>
       <c r="B63" t="s">
-        <v>101</v>
+        <v>147</v>
       </c>
       <c r="C63" t="s">
-        <v>102</v>
+        <v>148</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -1616,10 +1622,10 @@
         <v>10</v>
       </c>
       <c r="B64" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="C64" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -1627,10 +1633,10 @@
         <v>10</v>
       </c>
       <c r="B65" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C65" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -1638,10 +1644,10 @@
         <v>10</v>
       </c>
       <c r="B66" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C66" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -1649,10 +1655,10 @@
         <v>10</v>
       </c>
       <c r="B67" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -1660,10 +1666,10 @@
         <v>10</v>
       </c>
       <c r="B68" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C68" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -1671,10 +1677,10 @@
         <v>10</v>
       </c>
       <c r="B69" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C69" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -1682,10 +1688,10 @@
         <v>10</v>
       </c>
       <c r="B70" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C70" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -1693,10 +1699,10 @@
         <v>10</v>
       </c>
       <c r="B71" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C71" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -1704,10 +1710,10 @@
         <v>10</v>
       </c>
       <c r="B72" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C72" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -1715,10 +1721,10 @@
         <v>10</v>
       </c>
       <c r="B73" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C73" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -1726,10 +1732,10 @@
         <v>10</v>
       </c>
       <c r="B74" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="C74" t="s">
-        <v>134</v>
+        <v>112</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -1737,10 +1743,10 @@
         <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C75" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -1748,10 +1754,10 @@
         <v>10</v>
       </c>
       <c r="B76" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="C76" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -1759,10 +1765,10 @@
         <v>10</v>
       </c>
       <c r="B77" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C77" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -1770,10 +1776,10 @@
         <v>10</v>
       </c>
       <c r="B78" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C78" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -1781,10 +1787,10 @@
         <v>10</v>
       </c>
       <c r="B79" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="C79" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -1792,10 +1798,10 @@
         <v>10</v>
       </c>
       <c r="B80" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C80" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -1803,10 +1809,10 @@
         <v>10</v>
       </c>
       <c r="B81" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C81" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -1814,10 +1820,10 @@
         <v>10</v>
       </c>
       <c r="B82" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C82" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -1825,10 +1831,10 @@
         <v>10</v>
       </c>
       <c r="B83" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C83" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -1836,10 +1842,10 @@
         <v>10</v>
       </c>
       <c r="B84" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C84" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -1847,10 +1853,10 @@
         <v>10</v>
       </c>
       <c r="B85" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C85" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -1858,10 +1864,10 @@
         <v>10</v>
       </c>
       <c r="B86" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C86" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -1869,10 +1875,10 @@
         <v>10</v>
       </c>
       <c r="B87" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C87" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -1880,10 +1886,10 @@
         <v>10</v>
       </c>
       <c r="B88" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C88" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -1891,10 +1897,10 @@
         <v>10</v>
       </c>
       <c r="B89" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C89" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -1902,10 +1908,10 @@
         <v>10</v>
       </c>
       <c r="B90" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C90" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -1913,15 +1919,26 @@
         <v>10</v>
       </c>
       <c r="B91" t="s">
+        <v>167</v>
+      </c>
+      <c r="C91" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>10</v>
+      </c>
+      <c r="B92" t="s">
         <v>169</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C92" t="s">
         <v>170</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C54">
-    <sortCondition ref="A2:A54"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C55">
+    <sortCondition ref="A2:A55"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Wszystko działa. Cache cały zrefaktoryzowany. Kody pocztowe się wczytują. Poszukwianie pojedyncze działa na standardowym algorytmie. Jeszcze 170 błędów PNA
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B398410F-E4FC-4CC8-B132-F28FF3A22816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E29DCD5F-E8C3-4366-AE75-E8C30CD29B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="199">
   <si>
     <t>KEN</t>
   </si>
@@ -483,9 +494,6 @@
     <t>P.por.</t>
   </si>
   <si>
-    <t>podporucznik</t>
-  </si>
-  <si>
     <t>bpa</t>
   </si>
   <si>
@@ -544,6 +552,87 @@
   </si>
   <si>
     <t>Bohaterów Warszawy</t>
+  </si>
+  <si>
+    <t>Frycza-Modrzewskiego</t>
+  </si>
+  <si>
+    <t>Frycza Modrzewskiego</t>
+  </si>
+  <si>
+    <t>*Armii Wojska Polskiego</t>
+  </si>
+  <si>
+    <t>Ludwika van_Beethovena</t>
+  </si>
+  <si>
+    <t>Ludwika*Beethovena</t>
+  </si>
+  <si>
+    <t>Chełmońskiego-Deptak</t>
+  </si>
+  <si>
+    <t>Chełmońskiego*Deptak</t>
+  </si>
+  <si>
+    <t>*Wojska Polskiego</t>
+  </si>
+  <si>
+    <t>-Pseudonim</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>20-tu</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Picasso</t>
+  </si>
+  <si>
+    <t>Picassa</t>
+  </si>
+  <si>
+    <t>Pablo*Picasso</t>
+  </si>
+  <si>
+    <t>Pabla*Picassa</t>
+  </si>
+  <si>
+    <t>podporucznika</t>
+  </si>
+  <si>
+    <t>Jana*Bosko</t>
+  </si>
+  <si>
+    <t>Jana*Bosco</t>
+  </si>
+  <si>
+    <t>Boduena</t>
+  </si>
+  <si>
+    <t>Badouina</t>
+  </si>
+  <si>
+    <t>!*AWP</t>
+  </si>
+  <si>
+    <t>!*WP</t>
+  </si>
+  <si>
+    <t>Kaden-</t>
+  </si>
+  <si>
+    <t>Kadena-</t>
+  </si>
+  <si>
+    <t>WOPR</t>
+  </si>
+  <si>
+    <t>Wodnego Ochotniczego Pogotowia Ratunkowego</t>
   </si>
 </sst>
 </file>
@@ -917,7 +1006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.28515625" customWidth="1"/>
@@ -1303,10 +1392,10 @@
         <v>10</v>
       </c>
       <c r="B35" t="s">
+        <v>170</v>
+      </c>
+      <c r="C35" t="s">
         <v>171</v>
-      </c>
-      <c r="C35" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1834,7 +1923,7 @@
         <v>151</v>
       </c>
       <c r="C83" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -1842,10 +1931,10 @@
         <v>10</v>
       </c>
       <c r="B84" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C84" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -1853,10 +1942,10 @@
         <v>10</v>
       </c>
       <c r="B85" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C85" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -1864,10 +1953,10 @@
         <v>10</v>
       </c>
       <c r="B86" t="s">
+        <v>153</v>
+      </c>
+      <c r="C86" t="s">
         <v>154</v>
-      </c>
-      <c r="C86" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -1875,10 +1964,10 @@
         <v>10</v>
       </c>
       <c r="B87" t="s">
+        <v>155</v>
+      </c>
+      <c r="C87" t="s">
         <v>156</v>
-      </c>
-      <c r="C87" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -1886,10 +1975,10 @@
         <v>10</v>
       </c>
       <c r="B88" t="s">
+        <v>157</v>
+      </c>
+      <c r="C88" t="s">
         <v>158</v>
-      </c>
-      <c r="C88" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -1897,10 +1986,10 @@
         <v>10</v>
       </c>
       <c r="B89" t="s">
+        <v>162</v>
+      </c>
+      <c r="C89" t="s">
         <v>163</v>
-      </c>
-      <c r="C89" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -1908,10 +1997,10 @@
         <v>10</v>
       </c>
       <c r="B90" t="s">
+        <v>164</v>
+      </c>
+      <c r="C90" t="s">
         <v>165</v>
-      </c>
-      <c r="C90" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -1919,10 +2008,10 @@
         <v>10</v>
       </c>
       <c r="B91" t="s">
+        <v>166</v>
+      </c>
+      <c r="C91" t="s">
         <v>167</v>
-      </c>
-      <c r="C91" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -1930,10 +2019,164 @@
         <v>10</v>
       </c>
       <c r="B92" t="s">
+        <v>168</v>
+      </c>
+      <c r="C92" t="s">
         <v>169</v>
       </c>
-      <c r="C92" t="s">
-        <v>170</v>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>10</v>
+      </c>
+      <c r="B93" t="s">
+        <v>172</v>
+      </c>
+      <c r="C93" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>10</v>
+      </c>
+      <c r="B94" t="s">
+        <v>193</v>
+      </c>
+      <c r="C94" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>10</v>
+      </c>
+      <c r="B95" t="s">
+        <v>176</v>
+      </c>
+      <c r="C95" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>10</v>
+      </c>
+      <c r="B96" t="s">
+        <v>157</v>
+      </c>
+      <c r="C96" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>10</v>
+      </c>
+      <c r="B97" t="s">
+        <v>177</v>
+      </c>
+      <c r="C97" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>10</v>
+      </c>
+      <c r="B98" t="s">
+        <v>194</v>
+      </c>
+      <c r="C98" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>10</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C99" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>10</v>
+      </c>
+      <c r="B100" t="s">
+        <v>182</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>10</v>
+      </c>
+      <c r="B101" t="s">
+        <v>184</v>
+      </c>
+      <c r="C101" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>10</v>
+      </c>
+      <c r="B102" t="s">
+        <v>195</v>
+      </c>
+      <c r="C102" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>10</v>
+      </c>
+      <c r="B103" t="s">
+        <v>186</v>
+      </c>
+      <c r="C103" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>10</v>
+      </c>
+      <c r="B104" t="s">
+        <v>189</v>
+      </c>
+      <c r="C104" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>10</v>
+      </c>
+      <c r="B105" t="s">
+        <v>191</v>
+      </c>
+      <c r="C105" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>10</v>
+      </c>
+      <c r="B106" t="s">
+        <v>197</v>
+      </c>
+      <c r="C106" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Usunięta część błędów PNA
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E29DCD5F-E8C3-4366-AE75-E8C30CD29B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77041DCA-3CBB-4598-A52A-9770D94E6F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="215">
   <si>
     <t>KEN</t>
   </si>
@@ -623,16 +623,64 @@
     <t>!*WP</t>
   </si>
   <si>
-    <t>Kaden-</t>
-  </si>
-  <si>
-    <t>Kadena-</t>
-  </si>
-  <si>
     <t>WOPR</t>
   </si>
   <si>
     <t>Wodnego Ochotniczego Pogotowia Ratunkowego</t>
+  </si>
+  <si>
+    <t>Gwardii Ludowej WRN</t>
+  </si>
+  <si>
+    <t>Gwardii Ludowej Wolność Równość Niepodległość</t>
+  </si>
+  <si>
+    <t>Misjonarzy Oblatów MN</t>
+  </si>
+  <si>
+    <t>Misjonarzy Oblatów Marii Niepokalanej</t>
+  </si>
+  <si>
+    <t>Grzmot-Skotnickiego</t>
+  </si>
+  <si>
+    <t>Grzmota-Skotnickiego</t>
+  </si>
+  <si>
+    <t>Waltera-Janke</t>
+  </si>
+  <si>
+    <t>Waltera-Jankego</t>
+  </si>
+  <si>
+    <t>Heyki</t>
+  </si>
+  <si>
+    <t>Heykego</t>
+  </si>
+  <si>
+    <t>Kaden-Bandrowskiego</t>
+  </si>
+  <si>
+    <t>Kadena-Bandrowskiego</t>
+  </si>
+  <si>
+    <t>Hauke-Bosaka</t>
+  </si>
+  <si>
+    <t>Haukego-Bosaka</t>
+  </si>
+  <si>
+    <t>Dunin-Wąsowicza</t>
+  </si>
+  <si>
+    <t>Dunina-Wąsowicza</t>
+  </si>
+  <si>
+    <t>Boj. o Wolność i Demokrację</t>
+  </si>
+  <si>
+    <t>Bojowników o Wolność i Demokrację</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.28515625" customWidth="1"/>
@@ -1975,10 +2023,10 @@
         <v>10</v>
       </c>
       <c r="B88" t="s">
-        <v>157</v>
+        <v>209</v>
       </c>
       <c r="C88" t="s">
-        <v>158</v>
+        <v>210</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -2129,10 +2177,10 @@
         <v>10</v>
       </c>
       <c r="B102" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
       <c r="C102" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
@@ -2140,10 +2188,10 @@
         <v>10</v>
       </c>
       <c r="B103" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
       <c r="C103" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
@@ -2151,10 +2199,10 @@
         <v>10</v>
       </c>
       <c r="B104" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C104" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
@@ -2162,10 +2210,10 @@
         <v>10</v>
       </c>
       <c r="B105" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C105" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
@@ -2173,10 +2221,87 @@
         <v>10</v>
       </c>
       <c r="B106" t="s">
+        <v>191</v>
+      </c>
+      <c r="C106" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>10</v>
+      </c>
+      <c r="B107" t="s">
+        <v>195</v>
+      </c>
+      <c r="C107" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>10</v>
+      </c>
+      <c r="B108" t="s">
         <v>197</v>
       </c>
-      <c r="C106" t="s">
+      <c r="C108" t="s">
         <v>198</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>10</v>
+      </c>
+      <c r="B109" t="s">
+        <v>199</v>
+      </c>
+      <c r="C109" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>10</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>10</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>10</v>
+      </c>
+      <c r="B112" t="s">
+        <v>205</v>
+      </c>
+      <c r="C112" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>10</v>
+      </c>
+      <c r="B113" t="s">
+        <v>213</v>
+      </c>
+      <c r="C113" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Całe PNA obrobione, została tylko ulica Spokojna W Ostrowie Mazowieckim
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B03078BB-C2CC-4C3C-8475-CCE5A9B44A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1FBB654-2EFF-4177-8E1F-63A9E45B37FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="228">
   <si>
     <t>KEN</t>
   </si>
@@ -708,6 +708,18 @@
   </si>
   <si>
     <t>Czesława Hake</t>
+  </si>
+  <si>
+    <t>Eliasza Proroka</t>
+  </si>
+  <si>
+    <t>proroka Eliasza</t>
+  </si>
+  <si>
+    <t>Tagore</t>
+  </si>
+  <si>
+    <t>Tagore'a</t>
   </si>
 </sst>
 </file>
@@ -1081,7 +1093,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.28515625" customWidth="1"/>
@@ -2397,6 +2409,28 @@
         <v>222</v>
       </c>
     </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>10</v>
+      </c>
+      <c r="B120" t="s">
+        <v>224</v>
+      </c>
+      <c r="C120" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>10</v>
+      </c>
+      <c r="B121" t="s">
+        <v>226</v>
+      </c>
+      <c r="C121" t="s">
+        <v>227</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C55">
     <sortCondition ref="A2:A55"/>

</xml_diff>

<commit_message>
Zostało 8 błędów w PNA
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1FBB654-2EFF-4177-8E1F-63A9E45B37FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCA7DE9-D965-45CE-9F1D-F7383712AFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="233">
   <si>
     <t>KEN</t>
   </si>
@@ -720,6 +720,21 @@
   </si>
   <si>
     <t>Tagore'a</t>
+  </si>
+  <si>
+    <t>!-go*</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>pl. Rynek</t>
+  </si>
+  <si>
+    <t>Rynek</t>
+  </si>
+  <si>
+    <t>pl.Rynek</t>
   </si>
 </sst>
 </file>
@@ -1093,7 +1108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C124"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.28515625" customWidth="1"/>
@@ -2431,6 +2446,39 @@
         <v>227</v>
       </c>
     </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>10</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C122" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>10</v>
+      </c>
+      <c r="B123" t="s">
+        <v>230</v>
+      </c>
+      <c r="C123" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>10</v>
+      </c>
+      <c r="B124" t="s">
+        <v>232</v>
+      </c>
+      <c r="C124" t="s">
+        <v>231</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C55">
     <sortCondition ref="A2:A55"/>

</xml_diff>

<commit_message>
Został już tylko plac Katedralny w Łodzi jeśli chodzi o błędy PNA
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCA7DE9-D965-45CE-9F1D-F7383712AFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0173E72-D999-497C-8DD7-71AA4511EEEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -716,25 +716,25 @@
     <t>proroka Eliasza</t>
   </si>
   <si>
+    <t>!-go*</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>pl. Rynek</t>
+  </si>
+  <si>
+    <t>Rynek</t>
+  </si>
+  <si>
+    <t>pl.Rynek</t>
+  </si>
+  <si>
     <t>Tagore</t>
   </si>
   <si>
     <t>Tagore'a</t>
-  </si>
-  <si>
-    <t>!-go*</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>pl. Rynek</t>
-  </si>
-  <si>
-    <t>Rynek</t>
-  </si>
-  <si>
-    <t>pl.Rynek</t>
   </si>
 </sst>
 </file>
@@ -2440,10 +2440,10 @@
         <v>10</v>
       </c>
       <c r="B121" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="C121" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
@@ -2451,10 +2451,10 @@
         <v>10</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C122" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
@@ -2462,10 +2462,10 @@
         <v>10</v>
       </c>
       <c r="B123" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C123" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
@@ -2473,10 +2473,10 @@
         <v>10</v>
       </c>
       <c r="B124" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C124" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ogólnie działa, dodałem pseudonimy. 131 błędów PNA, merytorycznych.
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC09171-8613-43B2-BBE3-D1C5008555B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64452333-53BD-475B-A537-1D3CE6D3A50A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1957,10 +1957,10 @@
         <v>10</v>
       </c>
       <c r="B76" t="s">
+        <v>128</v>
+      </c>
+      <c r="C76" t="s">
         <v>127</v>
-      </c>
-      <c r="C76" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Poprawki SAP działają, około 1500 błędów
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A640746-DF6D-4466-8092-E6CD40FDD20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEB62BBC-4524-4A4B-8C16-C95BC2E10C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="2835" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="424">
   <si>
     <t>KEN</t>
   </si>
@@ -1275,6 +1275,39 @@
   </si>
   <si>
     <t>Prezydenta Rzeczpospolitej Polskiej</t>
+  </si>
+  <si>
+    <t>Dunin Wąsowicza</t>
+  </si>
+  <si>
+    <t>Dunin-Wasowicza</t>
+  </si>
+  <si>
+    <t>Drugiego Pułku</t>
+  </si>
+  <si>
+    <t>2 Pułku</t>
+  </si>
+  <si>
+    <t>Hauke Bosaka</t>
+  </si>
+  <si>
+    <t>Zamoyskiego</t>
+  </si>
+  <si>
+    <t>Zamojskiego</t>
+  </si>
+  <si>
+    <t>Zamoyskiej</t>
+  </si>
+  <si>
+    <t>Zamojskiej</t>
+  </si>
+  <si>
+    <t>Zamoyskich</t>
+  </si>
+  <si>
+    <t>Zamojskich</t>
   </si>
 </sst>
 </file>
@@ -1648,7 +1681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C218"/>
+  <dimension ref="A1:C225"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="35.85546875" customWidth="1"/>
@@ -1671,10 +1704,10 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1682,10 +1715,10 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1693,10 +1726,10 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1704,10 +1737,10 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1715,10 +1748,10 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1726,10 +1759,10 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1737,10 +1770,10 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1748,10 +1781,10 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1759,10 +1792,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1770,10 +1803,10 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -1781,10 +1814,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1792,10 +1825,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1803,10 +1836,10 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>73</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -1825,10 +1858,10 @@
         <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1836,10 +1869,10 @@
         <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1847,10 +1880,10 @@
         <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1858,10 +1891,10 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C19" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1869,10 +1902,10 @@
         <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1880,32 +1913,32 @@
         <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>10</v>
       </c>
-      <c r="B22" t="s">
-        <v>0</v>
+      <c r="B22" s="1" t="s">
+        <v>93</v>
       </c>
       <c r="C22" t="s">
-        <v>1</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>10</v>
       </c>
-      <c r="B23" t="s">
-        <v>4</v>
+      <c r="B23" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="C23" t="s">
-        <v>1</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1913,10 +1946,10 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>5</v>
+        <v>181</v>
       </c>
       <c r="C24" t="s">
-        <v>6</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1924,10 +1957,10 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>15</v>
+        <v>125</v>
       </c>
       <c r="C25" t="s">
-        <v>14</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1935,10 +1968,10 @@
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>24</v>
+        <v>99</v>
       </c>
       <c r="C26" t="s">
-        <v>25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1946,10 +1979,10 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>26</v>
+        <v>143</v>
       </c>
       <c r="C27" t="s">
-        <v>27</v>
+        <v>144</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1957,10 +1990,10 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>2</v>
+        <v>101</v>
       </c>
       <c r="C28" t="s">
-        <v>3</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1968,10 +2001,10 @@
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>16</v>
+        <v>133</v>
       </c>
       <c r="C29" t="s">
-        <v>17</v>
+        <v>134</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1979,10 +2012,10 @@
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" t="s">
-        <v>19</v>
+        <v>95</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1990,10 +2023,10 @@
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>137</v>
-      </c>
-      <c r="C31" t="s">
-        <v>138</v>
+        <v>96</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -2001,10 +2034,10 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>135</v>
+        <v>97</v>
       </c>
       <c r="C32" t="s">
-        <v>136</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -2012,10 +2045,10 @@
         <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="C33" t="s">
-        <v>21</v>
+        <v>124</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -2023,10 +2056,10 @@
         <v>10</v>
       </c>
       <c r="B34" t="s">
-        <v>23</v>
+        <v>182</v>
       </c>
       <c r="C34" t="s">
-        <v>22</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -2034,10 +2067,10 @@
         <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>162</v>
-      </c>
-      <c r="C35" t="s">
-        <v>163</v>
+        <v>94</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -2045,10 +2078,10 @@
         <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>41</v>
+        <v>113</v>
       </c>
       <c r="C36" t="s">
-        <v>42</v>
+        <v>103</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -2056,32 +2089,32 @@
         <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>43</v>
+        <v>114</v>
       </c>
       <c r="C37" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>92</v>
+      <c r="B38" t="s">
+        <v>115</v>
       </c>
       <c r="C38" t="s">
-        <v>49</v>
+        <v>105</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>10</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>93</v>
+      <c r="B39" t="s">
+        <v>116</v>
       </c>
       <c r="C39" t="s">
-        <v>49</v>
+        <v>106</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -2089,10 +2122,10 @@
         <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>94</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>50</v>
+        <v>117</v>
+      </c>
+      <c r="C40" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -2100,10 +2133,10 @@
         <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>95</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>50</v>
+        <v>118</v>
+      </c>
+      <c r="C41" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -2111,10 +2144,10 @@
         <v>10</v>
       </c>
       <c r="B42" t="s">
-        <v>96</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>50</v>
+        <v>119</v>
+      </c>
+      <c r="C42" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -2122,10 +2155,10 @@
         <v>10</v>
       </c>
       <c r="B43" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
       <c r="C43" t="s">
-        <v>52</v>
+        <v>110</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -2133,10 +2166,10 @@
         <v>10</v>
       </c>
       <c r="B44" t="s">
-        <v>55</v>
+        <v>121</v>
       </c>
       <c r="C44" t="s">
-        <v>52</v>
+        <v>111</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -2144,21 +2177,21 @@
         <v>10</v>
       </c>
       <c r="B45" t="s">
-        <v>53</v>
+        <v>122</v>
       </c>
       <c r="C45" t="s">
-        <v>54</v>
+        <v>112</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>10</v>
       </c>
-      <c r="B46" t="s">
-        <v>25</v>
+      <c r="B46" s="1" t="s">
+        <v>225</v>
       </c>
       <c r="C46" t="s">
-        <v>54</v>
+        <v>226</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -2166,10 +2199,10 @@
         <v>10</v>
       </c>
       <c r="B47" t="s">
-        <v>27</v>
-      </c>
-      <c r="C47" t="s">
-        <v>56</v>
+        <v>171</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -2177,10 +2210,10 @@
         <v>10</v>
       </c>
       <c r="B48" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="C48" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -2188,10 +2221,10 @@
         <v>10</v>
       </c>
       <c r="B49" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="C49" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -2199,10 +2232,10 @@
         <v>10</v>
       </c>
       <c r="B50" t="s">
-        <v>57</v>
+        <v>286</v>
       </c>
       <c r="C50" t="s">
-        <v>58</v>
+        <v>287</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -2210,10 +2243,10 @@
         <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>59</v>
+        <v>282</v>
       </c>
       <c r="C51" t="s">
-        <v>60</v>
+        <v>283</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -2221,10 +2254,10 @@
         <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>47</v>
+        <v>241</v>
       </c>
       <c r="C52" t="s">
-        <v>48</v>
+        <v>242</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -2232,10 +2265,10 @@
         <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>45</v>
+        <v>220</v>
       </c>
       <c r="C53" t="s">
-        <v>46</v>
+        <v>219</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -2243,10 +2276,10 @@
         <v>10</v>
       </c>
       <c r="B54" t="s">
-        <v>85</v>
+        <v>160</v>
       </c>
       <c r="C54" t="s">
-        <v>86</v>
+        <v>161</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -2254,10 +2287,10 @@
         <v>10</v>
       </c>
       <c r="B55" t="s">
-        <v>91</v>
+        <v>300</v>
       </c>
       <c r="C55" t="s">
-        <v>22</v>
+        <v>301</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -2265,10 +2298,10 @@
         <v>10</v>
       </c>
       <c r="B56" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="C56" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -2276,10 +2309,10 @@
         <v>10</v>
       </c>
       <c r="B57" t="s">
-        <v>87</v>
+        <v>180</v>
       </c>
       <c r="C57" t="s">
-        <v>88</v>
+        <v>207</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -2287,10 +2320,10 @@
         <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>89</v>
+        <v>162</v>
       </c>
       <c r="C58" t="s">
-        <v>90</v>
+        <v>163</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -2298,10 +2331,10 @@
         <v>10</v>
       </c>
       <c r="B59" t="s">
-        <v>123</v>
+        <v>201</v>
       </c>
       <c r="C59" t="s">
-        <v>124</v>
+        <v>202</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -2309,10 +2342,10 @@
         <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>97</v>
+        <v>146</v>
       </c>
       <c r="C60" t="s">
-        <v>98</v>
+        <v>153</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -2320,10 +2353,10 @@
         <v>10</v>
       </c>
       <c r="B61" t="s">
-        <v>99</v>
+        <v>236</v>
       </c>
       <c r="C61" t="s">
-        <v>100</v>
+        <v>237</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -2331,10 +2364,10 @@
         <v>10</v>
       </c>
       <c r="B62" t="s">
-        <v>125</v>
+        <v>168</v>
       </c>
       <c r="C62" t="s">
-        <v>126</v>
+        <v>169</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -2342,10 +2375,10 @@
         <v>10</v>
       </c>
       <c r="B63" t="s">
-        <v>133</v>
+        <v>284</v>
       </c>
       <c r="C63" t="s">
-        <v>134</v>
+        <v>285</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -2353,10 +2386,10 @@
         <v>10</v>
       </c>
       <c r="B64" t="s">
-        <v>143</v>
+        <v>349</v>
       </c>
       <c r="C64" t="s">
-        <v>144</v>
+        <v>350</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -2364,10 +2397,10 @@
         <v>10</v>
       </c>
       <c r="B65" t="s">
-        <v>101</v>
+        <v>263</v>
       </c>
       <c r="C65" t="s">
-        <v>102</v>
+        <v>235</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -2375,10 +2408,10 @@
         <v>10</v>
       </c>
       <c r="B66" t="s">
-        <v>113</v>
+        <v>234</v>
       </c>
       <c r="C66" t="s">
-        <v>103</v>
+        <v>235</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -2386,10 +2419,10 @@
         <v>10</v>
       </c>
       <c r="B67" t="s">
-        <v>114</v>
+        <v>222</v>
       </c>
       <c r="C67" t="s">
-        <v>104</v>
+        <v>221</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -2397,10 +2430,10 @@
         <v>10</v>
       </c>
       <c r="B68" t="s">
-        <v>115</v>
+        <v>361</v>
       </c>
       <c r="C68" t="s">
-        <v>105</v>
+        <v>373</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -2408,10 +2441,10 @@
         <v>10</v>
       </c>
       <c r="B69" t="s">
-        <v>116</v>
+        <v>330</v>
       </c>
       <c r="C69" t="s">
-        <v>106</v>
+        <v>331</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -2419,10 +2452,10 @@
         <v>10</v>
       </c>
       <c r="B70" t="s">
-        <v>117</v>
+        <v>203</v>
       </c>
       <c r="C70" t="s">
-        <v>107</v>
+        <v>204</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -2430,10 +2463,10 @@
         <v>10</v>
       </c>
       <c r="B71" t="s">
-        <v>118</v>
+        <v>152</v>
       </c>
       <c r="C71" t="s">
-        <v>108</v>
+        <v>151</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -2441,10 +2474,10 @@
         <v>10</v>
       </c>
       <c r="B72" t="s">
-        <v>119</v>
+        <v>415</v>
       </c>
       <c r="C72" t="s">
-        <v>109</v>
+        <v>416</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -2452,10 +2485,10 @@
         <v>10</v>
       </c>
       <c r="B73" t="s">
-        <v>120</v>
+        <v>293</v>
       </c>
       <c r="C73" t="s">
-        <v>110</v>
+        <v>294</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -2463,10 +2496,10 @@
         <v>10</v>
       </c>
       <c r="B74" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="C74" t="s">
-        <v>111</v>
+        <v>140</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -2474,10 +2507,10 @@
         <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>122</v>
+        <v>413</v>
       </c>
       <c r="C75" t="s">
-        <v>112</v>
+        <v>200</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -2485,10 +2518,10 @@
         <v>10</v>
       </c>
       <c r="B76" t="s">
-        <v>128</v>
+        <v>414</v>
       </c>
       <c r="C76" t="s">
-        <v>127</v>
+        <v>200</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -2496,7 +2529,10 @@
         <v>10</v>
       </c>
       <c r="B77" t="s">
-        <v>130</v>
+        <v>199</v>
+      </c>
+      <c r="C77" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -2504,7 +2540,10 @@
         <v>10</v>
       </c>
       <c r="B78" t="s">
-        <v>129</v>
+        <v>53</v>
+      </c>
+      <c r="C78" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -2512,10 +2551,10 @@
         <v>10</v>
       </c>
       <c r="B79" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C79" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -2523,10 +2562,10 @@
         <v>10</v>
       </c>
       <c r="B80" t="s">
-        <v>139</v>
+        <v>362</v>
       </c>
       <c r="C80" t="s">
-        <v>140</v>
+        <v>374</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -2534,10 +2573,10 @@
         <v>10</v>
       </c>
       <c r="B81" t="s">
-        <v>141</v>
+        <v>316</v>
       </c>
       <c r="C81" t="s">
-        <v>142</v>
+        <v>317</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -2545,10 +2584,10 @@
         <v>10</v>
       </c>
       <c r="B82" t="s">
-        <v>203</v>
+        <v>223</v>
       </c>
       <c r="C82" t="s">
-        <v>204</v>
+        <v>224</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -2556,10 +2595,10 @@
         <v>10</v>
       </c>
       <c r="B83" t="s">
-        <v>145</v>
+        <v>264</v>
       </c>
       <c r="C83" t="s">
-        <v>177</v>
+        <v>265</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -2567,10 +2606,10 @@
         <v>10</v>
       </c>
       <c r="B84" t="s">
-        <v>146</v>
+        <v>392</v>
       </c>
       <c r="C84" t="s">
-        <v>153</v>
+        <v>393</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -2578,10 +2617,10 @@
         <v>10</v>
       </c>
       <c r="B85" t="s">
-        <v>152</v>
+        <v>344</v>
       </c>
       <c r="C85" t="s">
-        <v>151</v>
+        <v>345</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -2589,10 +2628,10 @@
         <v>10</v>
       </c>
       <c r="B86" t="s">
-        <v>147</v>
+        <v>342</v>
       </c>
       <c r="C86" t="s">
-        <v>148</v>
+        <v>343</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -2600,10 +2639,10 @@
         <v>10</v>
       </c>
       <c r="B87" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C87" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -2611,10 +2650,10 @@
         <v>10</v>
       </c>
       <c r="B88" t="s">
-        <v>197</v>
+        <v>164</v>
       </c>
       <c r="C88" t="s">
-        <v>198</v>
+        <v>165</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -2622,10 +2661,10 @@
         <v>10</v>
       </c>
       <c r="B89" t="s">
-        <v>154</v>
+        <v>409</v>
       </c>
       <c r="C89" t="s">
-        <v>155</v>
+        <v>410</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -2633,10 +2672,10 @@
         <v>10</v>
       </c>
       <c r="B90" t="s">
-        <v>156</v>
+        <v>290</v>
       </c>
       <c r="C90" t="s">
-        <v>157</v>
+        <v>410</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -2644,10 +2683,10 @@
         <v>10</v>
       </c>
       <c r="B91" t="s">
-        <v>158</v>
+        <v>248</v>
       </c>
       <c r="C91" t="s">
-        <v>159</v>
+        <v>249</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -2655,10 +2694,10 @@
         <v>10</v>
       </c>
       <c r="B92" t="s">
-        <v>160</v>
+        <v>251</v>
       </c>
       <c r="C92" t="s">
-        <v>161</v>
+        <v>252</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
@@ -2666,10 +2705,10 @@
         <v>10</v>
       </c>
       <c r="B93" t="s">
-        <v>164</v>
+        <v>358</v>
       </c>
       <c r="C93" t="s">
-        <v>165</v>
+        <v>370</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -2677,10 +2716,10 @@
         <v>10</v>
       </c>
       <c r="B94" t="s">
-        <v>181</v>
+        <v>359</v>
       </c>
       <c r="C94" t="s">
-        <v>166</v>
+        <v>371</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
@@ -2688,10 +2727,10 @@
         <v>10</v>
       </c>
       <c r="B95" t="s">
-        <v>348</v>
+        <v>302</v>
       </c>
       <c r="C95" t="s">
-        <v>167</v>
+        <v>309</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
@@ -2699,21 +2738,21 @@
         <v>10</v>
       </c>
       <c r="B96" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="C96" t="s">
-        <v>198</v>
+        <v>250</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>10</v>
       </c>
-      <c r="B97" t="s">
-        <v>168</v>
-      </c>
-      <c r="C97" t="s">
-        <v>169</v>
+      <c r="B97" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
@@ -2721,21 +2760,21 @@
         <v>10</v>
       </c>
       <c r="B98" t="s">
-        <v>182</v>
+        <v>253</v>
       </c>
       <c r="C98" t="s">
-        <v>170</v>
+        <v>254</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>10</v>
       </c>
-      <c r="B99" s="1" t="s">
-        <v>205</v>
+      <c r="B99" t="s">
+        <v>185</v>
       </c>
       <c r="C99" t="s">
-        <v>206</v>
+        <v>186</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
@@ -2743,10 +2782,10 @@
         <v>10</v>
       </c>
       <c r="B100" t="s">
-        <v>171</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>172</v>
+        <v>255</v>
+      </c>
+      <c r="C100" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
@@ -2754,10 +2793,10 @@
         <v>10</v>
       </c>
       <c r="B101" t="s">
-        <v>173</v>
+        <v>353</v>
       </c>
       <c r="C101" t="s">
-        <v>174</v>
+        <v>354</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
@@ -2765,10 +2804,10 @@
         <v>10</v>
       </c>
       <c r="B102" t="s">
-        <v>199</v>
+        <v>417</v>
       </c>
       <c r="C102" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
@@ -2776,10 +2815,10 @@
         <v>10</v>
       </c>
       <c r="B103" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C103" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
@@ -2787,10 +2826,10 @@
         <v>10</v>
       </c>
       <c r="B104" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="C104" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
@@ -2798,10 +2837,10 @@
         <v>10</v>
       </c>
       <c r="B105" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="C105" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
@@ -2809,10 +2848,10 @@
         <v>10</v>
       </c>
       <c r="B106" t="s">
-        <v>180</v>
+        <v>334</v>
       </c>
       <c r="C106" t="s">
-        <v>207</v>
+        <v>335</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
@@ -2820,10 +2859,10 @@
         <v>10</v>
       </c>
       <c r="B107" t="s">
-        <v>183</v>
+        <v>304</v>
       </c>
       <c r="C107" t="s">
-        <v>184</v>
+        <v>307</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
@@ -2831,10 +2870,10 @@
         <v>10</v>
       </c>
       <c r="B108" t="s">
-        <v>185</v>
+        <v>407</v>
       </c>
       <c r="C108" t="s">
-        <v>186</v>
+        <v>408</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
@@ -2842,32 +2881,29 @@
         <v>10</v>
       </c>
       <c r="B109" t="s">
-        <v>187</v>
+        <v>398</v>
       </c>
       <c r="C109" t="s">
-        <v>188</v>
+        <v>382</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>10</v>
       </c>
-      <c r="B110" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="C110" s="1" t="s">
-        <v>192</v>
+      <c r="B110" t="s">
+        <v>41</v>
+      </c>
+      <c r="C110" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>10</v>
       </c>
-      <c r="B111" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="C111" s="1" t="s">
-        <v>190</v>
+      <c r="B111" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
@@ -2875,10 +2911,7 @@
         <v>10</v>
       </c>
       <c r="B112" t="s">
-        <v>193</v>
-      </c>
-      <c r="C112" t="s">
-        <v>194</v>
+        <v>129</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
@@ -2886,21 +2919,21 @@
         <v>10</v>
       </c>
       <c r="B113" t="s">
-        <v>201</v>
+        <v>259</v>
       </c>
       <c r="C113" t="s">
-        <v>202</v>
+        <v>260</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>10</v>
       </c>
-      <c r="B114" s="1" t="s">
-        <v>208</v>
+      <c r="B114" t="s">
+        <v>305</v>
       </c>
       <c r="C114" t="s">
-        <v>209</v>
+        <v>306</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
@@ -2908,10 +2941,10 @@
         <v>10</v>
       </c>
       <c r="B115" t="s">
-        <v>210</v>
+        <v>257</v>
       </c>
       <c r="C115" t="s">
-        <v>211</v>
+        <v>258</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
@@ -2919,21 +2952,21 @@
         <v>10</v>
       </c>
       <c r="B116" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C116" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>10</v>
       </c>
-      <c r="B117" t="s">
-        <v>214</v>
+      <c r="B117" s="1" t="s">
+        <v>208</v>
       </c>
       <c r="C117" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
@@ -2941,10 +2974,10 @@
         <v>10</v>
       </c>
       <c r="B118" t="s">
-        <v>215</v>
+        <v>379</v>
       </c>
       <c r="C118" t="s">
-        <v>216</v>
+        <v>378</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
@@ -2952,10 +2985,10 @@
         <v>10</v>
       </c>
       <c r="B119" t="s">
-        <v>217</v>
+        <v>368</v>
       </c>
       <c r="C119" t="s">
-        <v>218</v>
+        <v>378</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
@@ -2963,10 +2996,10 @@
         <v>10</v>
       </c>
       <c r="B120" t="s">
-        <v>220</v>
+        <v>357</v>
       </c>
       <c r="C120" t="s">
-        <v>219</v>
+        <v>363</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
@@ -2974,10 +3007,10 @@
         <v>10</v>
       </c>
       <c r="B121" t="s">
-        <v>222</v>
+        <v>178</v>
       </c>
       <c r="C121" t="s">
-        <v>221</v>
+        <v>179</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
@@ -2985,10 +3018,10 @@
         <v>10</v>
       </c>
       <c r="B122" t="s">
-        <v>223</v>
+        <v>246</v>
       </c>
       <c r="C122" t="s">
-        <v>224</v>
+        <v>247</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
@@ -2996,21 +3029,21 @@
         <v>10</v>
       </c>
       <c r="B123" t="s">
-        <v>230</v>
+        <v>383</v>
       </c>
       <c r="C123" t="s">
-        <v>231</v>
+        <v>384</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>10</v>
       </c>
-      <c r="B124" s="1" t="s">
-        <v>225</v>
+      <c r="B124" t="s">
+        <v>328</v>
       </c>
       <c r="C124" t="s">
-        <v>226</v>
+        <v>329</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
@@ -3018,10 +3051,10 @@
         <v>10</v>
       </c>
       <c r="B125" t="s">
-        <v>227</v>
+        <v>338</v>
       </c>
       <c r="C125" t="s">
-        <v>228</v>
+        <v>339</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
@@ -3029,10 +3062,10 @@
         <v>10</v>
       </c>
       <c r="B126" t="s">
-        <v>229</v>
+        <v>396</v>
       </c>
       <c r="C126" t="s">
-        <v>228</v>
+        <v>397</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
@@ -3040,10 +3073,10 @@
         <v>10</v>
       </c>
       <c r="B127" t="s">
-        <v>234</v>
+        <v>154</v>
       </c>
       <c r="C127" t="s">
-        <v>235</v>
+        <v>155</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
@@ -3051,10 +3084,10 @@
         <v>10</v>
       </c>
       <c r="B128" t="s">
-        <v>236</v>
+        <v>261</v>
       </c>
       <c r="C128" t="s">
-        <v>237</v>
+        <v>262</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
@@ -3062,10 +3095,10 @@
         <v>10</v>
       </c>
       <c r="B129" t="s">
-        <v>238</v>
+        <v>394</v>
       </c>
       <c r="C129" t="s">
-        <v>239</v>
+        <v>395</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
@@ -3073,10 +3106,10 @@
         <v>10</v>
       </c>
       <c r="B130" t="s">
-        <v>240</v>
+        <v>312</v>
       </c>
       <c r="C130" t="s">
-        <v>245</v>
+        <v>313</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
@@ -3084,10 +3117,10 @@
         <v>10</v>
       </c>
       <c r="B131" t="s">
-        <v>241</v>
+        <v>4</v>
       </c>
       <c r="C131" t="s">
-        <v>242</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -3095,10 +3128,10 @@
         <v>10</v>
       </c>
       <c r="B132" t="s">
-        <v>243</v>
+        <v>195</v>
       </c>
       <c r="C132" t="s">
-        <v>244</v>
+        <v>196</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
@@ -3106,10 +3139,10 @@
         <v>10</v>
       </c>
       <c r="B133" t="s">
-        <v>246</v>
+        <v>280</v>
       </c>
       <c r="C133" t="s">
-        <v>247</v>
+        <v>281</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
@@ -3117,10 +3150,10 @@
         <v>10</v>
       </c>
       <c r="B134" t="s">
-        <v>248</v>
+        <v>385</v>
       </c>
       <c r="C134" t="s">
-        <v>249</v>
+        <v>386</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
@@ -3128,10 +3161,10 @@
         <v>10</v>
       </c>
       <c r="B135" t="s">
-        <v>190</v>
+        <v>401</v>
       </c>
       <c r="C135" t="s">
-        <v>250</v>
+        <v>402</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
@@ -3139,10 +3172,10 @@
         <v>10</v>
       </c>
       <c r="B136" t="s">
-        <v>251</v>
+        <v>310</v>
       </c>
       <c r="C136" t="s">
-        <v>252</v>
+        <v>311</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
@@ -3150,10 +3183,10 @@
         <v>10</v>
       </c>
       <c r="B137" t="s">
-        <v>253</v>
+        <v>5</v>
       </c>
       <c r="C137" t="s">
-        <v>254</v>
+        <v>6</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
@@ -3161,10 +3194,10 @@
         <v>10</v>
       </c>
       <c r="B138" t="s">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="C138" t="s">
-        <v>256</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
@@ -3172,10 +3205,10 @@
         <v>10</v>
       </c>
       <c r="B139" t="s">
-        <v>257</v>
+        <v>326</v>
       </c>
       <c r="C139" t="s">
-        <v>258</v>
+        <v>327</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
@@ -3183,10 +3216,10 @@
         <v>10</v>
       </c>
       <c r="B140" t="s">
-        <v>259</v>
+        <v>131</v>
       </c>
       <c r="C140" t="s">
-        <v>260</v>
+        <v>132</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
@@ -3194,10 +3227,10 @@
         <v>10</v>
       </c>
       <c r="B141" t="s">
-        <v>261</v>
+        <v>212</v>
       </c>
       <c r="C141" t="s">
-        <v>262</v>
+        <v>213</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
@@ -3205,10 +3238,10 @@
         <v>10</v>
       </c>
       <c r="B142" t="s">
-        <v>263</v>
+        <v>399</v>
       </c>
       <c r="C142" t="s">
-        <v>235</v>
+        <v>400</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
@@ -3216,10 +3249,10 @@
         <v>10</v>
       </c>
       <c r="B143" t="s">
-        <v>264</v>
+        <v>388</v>
       </c>
       <c r="C143" t="s">
-        <v>265</v>
+        <v>389</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
@@ -3227,10 +3260,10 @@
         <v>10</v>
       </c>
       <c r="B144" t="s">
-        <v>266</v>
+        <v>387</v>
       </c>
       <c r="C144" t="s">
-        <v>267</v>
+        <v>389</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
@@ -3238,10 +3271,10 @@
         <v>10</v>
       </c>
       <c r="B145" t="s">
-        <v>268</v>
+        <v>375</v>
       </c>
       <c r="C145" t="s">
-        <v>269</v>
+        <v>369</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
@@ -3249,10 +3282,10 @@
         <v>10</v>
       </c>
       <c r="B146" t="s">
-        <v>270</v>
+        <v>348</v>
       </c>
       <c r="C146" t="s">
-        <v>271</v>
+        <v>167</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
@@ -3260,10 +3293,10 @@
         <v>10</v>
       </c>
       <c r="B147" t="s">
-        <v>272</v>
+        <v>346</v>
       </c>
       <c r="C147" t="s">
-        <v>273</v>
+        <v>347</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
@@ -3271,10 +3304,10 @@
         <v>10</v>
       </c>
       <c r="B148" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="C148" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
@@ -3282,10 +3315,10 @@
         <v>10</v>
       </c>
       <c r="B149" t="s">
-        <v>274</v>
+        <v>380</v>
       </c>
       <c r="C149" t="s">
-        <v>275</v>
+        <v>381</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
@@ -3293,10 +3326,10 @@
         <v>10</v>
       </c>
       <c r="B150" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="C150" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
@@ -3315,10 +3348,10 @@
         <v>10</v>
       </c>
       <c r="B152" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="C152" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
@@ -3326,10 +3359,10 @@
         <v>10</v>
       </c>
       <c r="B153" t="s">
-        <v>280</v>
+        <v>141</v>
       </c>
       <c r="C153" t="s">
-        <v>281</v>
+        <v>142</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
@@ -3337,10 +3370,10 @@
         <v>10</v>
       </c>
       <c r="B154" t="s">
-        <v>288</v>
+        <v>187</v>
       </c>
       <c r="C154" t="s">
-        <v>289</v>
+        <v>188</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
@@ -3348,10 +3381,10 @@
         <v>10</v>
       </c>
       <c r="B155" t="s">
-        <v>282</v>
+        <v>403</v>
       </c>
       <c r="C155" t="s">
-        <v>283</v>
+        <v>404</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
@@ -3359,10 +3392,10 @@
         <v>10</v>
       </c>
       <c r="B156" t="s">
-        <v>284</v>
+        <v>268</v>
       </c>
       <c r="C156" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
@@ -3370,10 +3403,10 @@
         <v>10</v>
       </c>
       <c r="B157" t="s">
-        <v>286</v>
+        <v>270</v>
       </c>
       <c r="C157" t="s">
-        <v>287</v>
+        <v>271</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
@@ -3381,10 +3414,10 @@
         <v>10</v>
       </c>
       <c r="B158" t="s">
-        <v>291</v>
+        <v>272</v>
       </c>
       <c r="C158" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
@@ -3392,10 +3425,10 @@
         <v>10</v>
       </c>
       <c r="B159" t="s">
-        <v>293</v>
+        <v>2</v>
       </c>
       <c r="C159" t="s">
-        <v>294</v>
+        <v>3</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
@@ -3403,10 +3436,10 @@
         <v>10</v>
       </c>
       <c r="B160" t="s">
-        <v>295</v>
+        <v>158</v>
       </c>
       <c r="C160" t="s">
-        <v>296</v>
+        <v>159</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
@@ -3414,10 +3447,10 @@
         <v>10</v>
       </c>
       <c r="B161" t="s">
-        <v>297</v>
+        <v>149</v>
       </c>
       <c r="C161" t="s">
-        <v>296</v>
+        <v>150</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
@@ -3425,10 +3458,10 @@
         <v>10</v>
       </c>
       <c r="B162" t="s">
-        <v>298</v>
+        <v>314</v>
       </c>
       <c r="C162" t="s">
-        <v>299</v>
+        <v>315</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
@@ -3436,10 +3469,10 @@
         <v>10</v>
       </c>
       <c r="B163" t="s">
-        <v>300</v>
+        <v>20</v>
       </c>
       <c r="C163" t="s">
-        <v>301</v>
+        <v>21</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
@@ -3447,10 +3480,10 @@
         <v>10</v>
       </c>
       <c r="B164" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="C164" t="s">
-        <v>309</v>
+        <v>292</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
@@ -3458,10 +3491,10 @@
         <v>10</v>
       </c>
       <c r="B165" t="s">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="C165" t="s">
-        <v>308</v>
+        <v>289</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
@@ -3469,10 +3502,10 @@
         <v>10</v>
       </c>
       <c r="B166" t="s">
-        <v>304</v>
+        <v>318</v>
       </c>
       <c r="C166" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
@@ -3480,10 +3513,10 @@
         <v>10</v>
       </c>
       <c r="B167" t="s">
-        <v>305</v>
+        <v>145</v>
       </c>
       <c r="C167" t="s">
-        <v>306</v>
+        <v>177</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
@@ -3491,10 +3524,10 @@
         <v>10</v>
       </c>
       <c r="B168" t="s">
-        <v>310</v>
+        <v>360</v>
       </c>
       <c r="C168" t="s">
-        <v>311</v>
+        <v>372</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
@@ -3502,10 +3535,10 @@
         <v>10</v>
       </c>
       <c r="B169" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="C169" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
@@ -3513,10 +3546,10 @@
         <v>10</v>
       </c>
       <c r="B170" t="s">
-        <v>387</v>
+        <v>175</v>
       </c>
       <c r="C170" t="s">
-        <v>389</v>
+        <v>176</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
@@ -3524,10 +3557,10 @@
         <v>10</v>
       </c>
       <c r="B171" t="s">
-        <v>388</v>
+        <v>364</v>
       </c>
       <c r="C171" t="s">
-        <v>389</v>
+        <v>365</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
@@ -3535,10 +3568,10 @@
         <v>10</v>
       </c>
       <c r="B172" t="s">
-        <v>318</v>
+        <v>43</v>
       </c>
       <c r="C172" t="s">
-        <v>319</v>
+        <v>44</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
@@ -3546,10 +3579,10 @@
         <v>10</v>
       </c>
       <c r="B173" t="s">
-        <v>320</v>
+        <v>173</v>
       </c>
       <c r="C173" t="s">
-        <v>321</v>
+        <v>174</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
@@ -3557,10 +3590,10 @@
         <v>10</v>
       </c>
       <c r="B174" t="s">
-        <v>391</v>
+        <v>137</v>
       </c>
       <c r="C174" t="s">
-        <v>390</v>
+        <v>138</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
@@ -3568,10 +3601,10 @@
         <v>10</v>
       </c>
       <c r="B175" t="s">
-        <v>322</v>
+        <v>51</v>
       </c>
       <c r="C175" t="s">
-        <v>323</v>
+        <v>52</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
@@ -3579,10 +3612,10 @@
         <v>10</v>
       </c>
       <c r="B176" t="s">
-        <v>324</v>
+        <v>227</v>
       </c>
       <c r="C176" t="s">
-        <v>325</v>
+        <v>228</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
@@ -3590,10 +3623,10 @@
         <v>10</v>
       </c>
       <c r="B177" t="s">
-        <v>326</v>
+        <v>229</v>
       </c>
       <c r="C177" t="s">
-        <v>327</v>
+        <v>228</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
@@ -3601,10 +3634,10 @@
         <v>10</v>
       </c>
       <c r="B178" t="s">
-        <v>328</v>
+        <v>232</v>
       </c>
       <c r="C178" t="s">
-        <v>329</v>
+        <v>233</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
@@ -3612,10 +3645,10 @@
         <v>10</v>
       </c>
       <c r="B179" t="s">
-        <v>330</v>
+        <v>16</v>
       </c>
       <c r="C179" t="s">
-        <v>331</v>
+        <v>17</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
@@ -3623,10 +3656,10 @@
         <v>10</v>
       </c>
       <c r="B180" t="s">
-        <v>332</v>
+        <v>18</v>
       </c>
       <c r="C180" t="s">
-        <v>333</v>
+        <v>19</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
@@ -3634,21 +3667,21 @@
         <v>10</v>
       </c>
       <c r="B181" t="s">
-        <v>334</v>
+        <v>412</v>
       </c>
       <c r="C181" t="s">
-        <v>335</v>
+        <v>411</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>10</v>
       </c>
-      <c r="B182" t="s">
-        <v>336</v>
+      <c r="B182" s="1" t="s">
+        <v>205</v>
       </c>
       <c r="C182" t="s">
-        <v>337</v>
+        <v>206</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
@@ -3656,10 +3689,10 @@
         <v>10</v>
       </c>
       <c r="B183" t="s">
-        <v>338</v>
+        <v>87</v>
       </c>
       <c r="C183" t="s">
-        <v>339</v>
+        <v>88</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
@@ -3667,10 +3700,10 @@
         <v>10</v>
       </c>
       <c r="B184" t="s">
-        <v>340</v>
+        <v>391</v>
       </c>
       <c r="C184" t="s">
-        <v>341</v>
+        <v>390</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
@@ -3678,10 +3711,10 @@
         <v>10</v>
       </c>
       <c r="B185" t="s">
-        <v>342</v>
+        <v>274</v>
       </c>
       <c r="C185" t="s">
-        <v>343</v>
+        <v>275</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
@@ -3689,10 +3722,10 @@
         <v>10</v>
       </c>
       <c r="B186" t="s">
-        <v>344</v>
+        <v>156</v>
       </c>
       <c r="C186" t="s">
-        <v>345</v>
+        <v>157</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
@@ -3700,10 +3733,10 @@
         <v>10</v>
       </c>
       <c r="B187" t="s">
-        <v>346</v>
+        <v>214</v>
       </c>
       <c r="C187" t="s">
-        <v>347</v>
+        <v>216</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
@@ -3711,10 +3744,10 @@
         <v>10</v>
       </c>
       <c r="B188" t="s">
-        <v>349</v>
+        <v>215</v>
       </c>
       <c r="C188" t="s">
-        <v>350</v>
+        <v>216</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
@@ -3722,10 +3755,10 @@
         <v>10</v>
       </c>
       <c r="B189" t="s">
-        <v>351</v>
+        <v>336</v>
       </c>
       <c r="C189" t="s">
-        <v>352</v>
+        <v>337</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
@@ -3733,10 +3766,10 @@
         <v>10</v>
       </c>
       <c r="B190" t="s">
-        <v>353</v>
+        <v>59</v>
       </c>
       <c r="C190" t="s">
-        <v>354</v>
+        <v>60</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
@@ -3744,10 +3777,10 @@
         <v>10</v>
       </c>
       <c r="B191" t="s">
-        <v>355</v>
+        <v>217</v>
       </c>
       <c r="C191" t="s">
-        <v>356</v>
+        <v>218</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
@@ -3755,10 +3788,10 @@
         <v>10</v>
       </c>
       <c r="B192" t="s">
-        <v>357</v>
+        <v>238</v>
       </c>
       <c r="C192" t="s">
-        <v>363</v>
+        <v>239</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
@@ -3766,10 +3799,10 @@
         <v>10</v>
       </c>
       <c r="B193" t="s">
-        <v>364</v>
+        <v>57</v>
       </c>
       <c r="C193" t="s">
-        <v>365</v>
+        <v>58</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
@@ -3777,10 +3810,10 @@
         <v>10</v>
       </c>
       <c r="B194" t="s">
-        <v>366</v>
+        <v>298</v>
       </c>
       <c r="C194" t="s">
-        <v>367</v>
+        <v>299</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
@@ -3788,10 +3821,10 @@
         <v>10</v>
       </c>
       <c r="B195" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="C195" t="s">
-        <v>382</v>
+        <v>46</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
@@ -3799,10 +3832,10 @@
         <v>10</v>
       </c>
       <c r="B196" t="s">
-        <v>379</v>
+        <v>332</v>
       </c>
       <c r="C196" t="s">
-        <v>378</v>
+        <v>333</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
@@ -3810,10 +3843,10 @@
         <v>10</v>
       </c>
       <c r="B197" t="s">
-        <v>368</v>
+        <v>89</v>
       </c>
       <c r="C197" t="s">
-        <v>378</v>
+        <v>90</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
@@ -3821,10 +3854,10 @@
         <v>10</v>
       </c>
       <c r="B198" t="s">
-        <v>375</v>
+        <v>355</v>
       </c>
       <c r="C198" t="s">
-        <v>369</v>
+        <v>356</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
@@ -3832,10 +3865,10 @@
         <v>10</v>
       </c>
       <c r="B199" t="s">
-        <v>358</v>
+        <v>230</v>
       </c>
       <c r="C199" t="s">
-        <v>370</v>
+        <v>231</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
@@ -3843,10 +3876,10 @@
         <v>10</v>
       </c>
       <c r="B200" t="s">
-        <v>359</v>
+        <v>297</v>
       </c>
       <c r="C200" t="s">
-        <v>371</v>
+        <v>296</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
@@ -3854,10 +3887,10 @@
         <v>10</v>
       </c>
       <c r="B201" t="s">
-        <v>360</v>
+        <v>295</v>
       </c>
       <c r="C201" t="s">
-        <v>372</v>
+        <v>296</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
@@ -3865,10 +3898,10 @@
         <v>10</v>
       </c>
       <c r="B202" t="s">
-        <v>361</v>
+        <v>278</v>
       </c>
       <c r="C202" t="s">
-        <v>373</v>
+        <v>279</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
@@ -3876,10 +3909,10 @@
         <v>10</v>
       </c>
       <c r="B203" t="s">
-        <v>362</v>
+        <v>62</v>
       </c>
       <c r="C203" t="s">
-        <v>374</v>
+        <v>61</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
@@ -3887,10 +3920,10 @@
         <v>10</v>
       </c>
       <c r="B204" t="s">
-        <v>383</v>
+        <v>47</v>
       </c>
       <c r="C204" t="s">
-        <v>384</v>
+        <v>48</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
@@ -3898,10 +3931,10 @@
         <v>10</v>
       </c>
       <c r="B205" t="s">
-        <v>376</v>
+        <v>135</v>
       </c>
       <c r="C205" t="s">
-        <v>377</v>
+        <v>136</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
@@ -3909,10 +3942,10 @@
         <v>10</v>
       </c>
       <c r="B206" t="s">
-        <v>380</v>
+        <v>366</v>
       </c>
       <c r="C206" t="s">
-        <v>381</v>
+        <v>367</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -3920,21 +3953,21 @@
         <v>10</v>
       </c>
       <c r="B207" t="s">
-        <v>385</v>
+        <v>351</v>
       </c>
       <c r="C207" t="s">
-        <v>386</v>
+        <v>352</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>10</v>
       </c>
-      <c r="B208" t="s">
-        <v>392</v>
-      </c>
-      <c r="C208" t="s">
-        <v>393</v>
+      <c r="B208" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C208" s="1" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
@@ -3942,10 +3975,10 @@
         <v>10</v>
       </c>
       <c r="B209" t="s">
-        <v>394</v>
+        <v>303</v>
       </c>
       <c r="C209" t="s">
-        <v>395</v>
+        <v>308</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
@@ -3953,10 +3986,10 @@
         <v>10</v>
       </c>
       <c r="B210" t="s">
-        <v>396</v>
+        <v>240</v>
       </c>
       <c r="C210" t="s">
-        <v>397</v>
+        <v>245</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
@@ -3964,10 +3997,10 @@
         <v>10</v>
       </c>
       <c r="B211" t="s">
-        <v>399</v>
+        <v>376</v>
       </c>
       <c r="C211" t="s">
-        <v>400</v>
+        <v>377</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
@@ -3975,10 +4008,10 @@
         <v>10</v>
       </c>
       <c r="B212" t="s">
-        <v>401</v>
+        <v>183</v>
       </c>
       <c r="C212" t="s">
-        <v>402</v>
+        <v>184</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
@@ -3986,10 +4019,10 @@
         <v>10</v>
       </c>
       <c r="B213" t="s">
-        <v>403</v>
+        <v>55</v>
       </c>
       <c r="C213" t="s">
-        <v>404</v>
+        <v>52</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
@@ -3997,10 +4030,10 @@
         <v>10</v>
       </c>
       <c r="B214" t="s">
-        <v>405</v>
+        <v>25</v>
       </c>
       <c r="C214" t="s">
-        <v>406</v>
+        <v>54</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
@@ -4008,10 +4041,10 @@
         <v>10</v>
       </c>
       <c r="B215" t="s">
-        <v>407</v>
+        <v>24</v>
       </c>
       <c r="C215" t="s">
-        <v>408</v>
+        <v>25</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
@@ -4019,10 +4052,10 @@
         <v>10</v>
       </c>
       <c r="B216" t="s">
-        <v>409</v>
+        <v>27</v>
       </c>
       <c r="C216" t="s">
-        <v>410</v>
+        <v>56</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
@@ -4030,10 +4063,10 @@
         <v>10</v>
       </c>
       <c r="B217" t="s">
-        <v>290</v>
+        <v>26</v>
       </c>
       <c r="C217" t="s">
-        <v>410</v>
+        <v>27</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
@@ -4041,15 +4074,93 @@
         <v>10</v>
       </c>
       <c r="B218" t="s">
-        <v>412</v>
+        <v>14</v>
       </c>
       <c r="C218" t="s">
-        <v>411</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>10</v>
+      </c>
+      <c r="B219" t="s">
+        <v>15</v>
+      </c>
+      <c r="C219" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>10</v>
+      </c>
+      <c r="B220" t="s">
+        <v>405</v>
+      </c>
+      <c r="C220" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>10</v>
+      </c>
+      <c r="B221" t="s">
+        <v>340</v>
+      </c>
+      <c r="C221" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>10</v>
+      </c>
+      <c r="B222" t="s">
+        <v>85</v>
+      </c>
+      <c r="C222" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>10</v>
+      </c>
+      <c r="B223" t="s">
+        <v>418</v>
+      </c>
+      <c r="C223" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>10</v>
+      </c>
+      <c r="B224" t="s">
+        <v>420</v>
+      </c>
+      <c r="C224" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>10</v>
+      </c>
+      <c r="B225" t="s">
+        <v>422</v>
+      </c>
+      <c r="C225" t="s">
+        <v>423</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C55">
-    <sortCondition ref="A2:A55"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C222">
+    <sortCondition ref="A2:A222"/>
+    <sortCondition ref="B2:B222"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Ustabilizowana sytuacja, 1100 błędów w SAP
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/KorektyNazw.xlsx
+++ b/TerytLoad/AppData/Updates/KorektyNazw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEB62BBC-4524-4A4B-8C16-C95BC2E10C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E06B2E7-F333-4AF0-9C31-E5174851B304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="428">
   <si>
     <t>KEN</t>
   </si>
@@ -1308,6 +1308,18 @@
   </si>
   <si>
     <t>Zamojskich</t>
+  </si>
+  <si>
+    <t>N.M.P.</t>
+  </si>
+  <si>
+    <t>Boh.Września</t>
+  </si>
+  <si>
+    <t>Bohaterów Września</t>
+  </si>
+  <si>
+    <t>Boh. Września</t>
   </si>
 </sst>
 </file>
@@ -1681,7 +1693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C225"/>
+  <dimension ref="A1:C228"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="35.85546875" customWidth="1"/>
@@ -3436,10 +3448,10 @@
         <v>10</v>
       </c>
       <c r="B160" t="s">
-        <v>158</v>
+        <v>424</v>
       </c>
       <c r="C160" t="s">
-        <v>159</v>
+        <v>3</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
@@ -3447,10 +3459,10 @@
         <v>10</v>
       </c>
       <c r="B161" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="C161" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
@@ -3458,10 +3470,10 @@
         <v>10</v>
       </c>
       <c r="B162" t="s">
-        <v>314</v>
+        <v>149</v>
       </c>
       <c r="C162" t="s">
-        <v>315</v>
+        <v>150</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
@@ -3469,10 +3481,10 @@
         <v>10</v>
       </c>
       <c r="B163" t="s">
-        <v>20</v>
+        <v>314</v>
       </c>
       <c r="C163" t="s">
-        <v>21</v>
+        <v>315</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
@@ -3480,10 +3492,10 @@
         <v>10</v>
       </c>
       <c r="B164" t="s">
-        <v>291</v>
+        <v>20</v>
       </c>
       <c r="C164" t="s">
-        <v>292</v>
+        <v>21</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
@@ -3491,10 +3503,10 @@
         <v>10</v>
       </c>
       <c r="B165" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C165" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
@@ -3502,10 +3514,10 @@
         <v>10</v>
       </c>
       <c r="B166" t="s">
-        <v>318</v>
+        <v>288</v>
       </c>
       <c r="C166" t="s">
-        <v>319</v>
+        <v>289</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
@@ -3513,10 +3525,10 @@
         <v>10</v>
       </c>
       <c r="B167" t="s">
-        <v>145</v>
+        <v>318</v>
       </c>
       <c r="C167" t="s">
-        <v>177</v>
+        <v>319</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
@@ -3524,10 +3536,10 @@
         <v>10</v>
       </c>
       <c r="B168" t="s">
-        <v>360</v>
+        <v>145</v>
       </c>
       <c r="C168" t="s">
-        <v>372</v>
+        <v>177</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
@@ -3535,10 +3547,10 @@
         <v>10</v>
       </c>
       <c r="B169" t="s">
-        <v>324</v>
+        <v>360</v>
       </c>
       <c r="C169" t="s">
-        <v>325</v>
+        <v>372</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
@@ -3546,10 +3558,10 @@
         <v>10</v>
       </c>
       <c r="B170" t="s">
-        <v>175</v>
+        <v>324</v>
       </c>
       <c r="C170" t="s">
-        <v>176</v>
+        <v>325</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
@@ -3557,10 +3569,10 @@
         <v>10</v>
       </c>
       <c r="B171" t="s">
-        <v>364</v>
+        <v>175</v>
       </c>
       <c r="C171" t="s">
-        <v>365</v>
+        <v>176</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
@@ -3568,10 +3580,10 @@
         <v>10</v>
       </c>
       <c r="B172" t="s">
-        <v>43</v>
+        <v>364</v>
       </c>
       <c r="C172" t="s">
-        <v>44</v>
+        <v>365</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
@@ -3579,10 +3591,10 @@
         <v>10</v>
       </c>
       <c r="B173" t="s">
-        <v>173</v>
+        <v>43</v>
       </c>
       <c r="C173" t="s">
-        <v>174</v>
+        <v>44</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
@@ -3590,10 +3602,10 @@
         <v>10</v>
       </c>
       <c r="B174" t="s">
-        <v>137</v>
+        <v>173</v>
       </c>
       <c r="C174" t="s">
-        <v>138</v>
+        <v>174</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
@@ -3601,10 +3613,10 @@
         <v>10</v>
       </c>
       <c r="B175" t="s">
-        <v>51</v>
+        <v>137</v>
       </c>
       <c r="C175" t="s">
-        <v>52</v>
+        <v>138</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
@@ -3612,10 +3624,10 @@
         <v>10</v>
       </c>
       <c r="B176" t="s">
-        <v>227</v>
+        <v>51</v>
       </c>
       <c r="C176" t="s">
-        <v>228</v>
+        <v>52</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
@@ -3623,7 +3635,7 @@
         <v>10</v>
       </c>
       <c r="B177" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C177" t="s">
         <v>228</v>
@@ -3634,10 +3646,10 @@
         <v>10</v>
       </c>
       <c r="B178" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C178" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
@@ -3645,10 +3657,10 @@
         <v>10</v>
       </c>
       <c r="B179" t="s">
-        <v>16</v>
+        <v>232</v>
       </c>
       <c r="C179" t="s">
-        <v>17</v>
+        <v>233</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
@@ -3656,10 +3668,10 @@
         <v>10</v>
       </c>
       <c r="B180" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C180" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
@@ -3667,32 +3679,32 @@
         <v>10</v>
       </c>
       <c r="B181" t="s">
-        <v>412</v>
+        <v>18</v>
       </c>
       <c r="C181" t="s">
-        <v>411</v>
+        <v>19</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>10</v>
       </c>
-      <c r="B182" s="1" t="s">
-        <v>205</v>
+      <c r="B182" t="s">
+        <v>412</v>
       </c>
       <c r="C182" t="s">
-        <v>206</v>
+        <v>411</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>10</v>
       </c>
-      <c r="B183" t="s">
-        <v>87</v>
+      <c r="B183" s="1" t="s">
+        <v>205</v>
       </c>
       <c r="C183" t="s">
-        <v>88</v>
+        <v>206</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
@@ -3700,10 +3712,10 @@
         <v>10</v>
       </c>
       <c r="B184" t="s">
-        <v>391</v>
+        <v>87</v>
       </c>
       <c r="C184" t="s">
-        <v>390</v>
+        <v>88</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
@@ -3711,10 +3723,10 @@
         <v>10</v>
       </c>
       <c r="B185" t="s">
-        <v>274</v>
+        <v>391</v>
       </c>
       <c r="C185" t="s">
-        <v>275</v>
+        <v>390</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
@@ -3722,10 +3734,10 @@
         <v>10</v>
       </c>
       <c r="B186" t="s">
-        <v>156</v>
+        <v>274</v>
       </c>
       <c r="C186" t="s">
-        <v>157</v>
+        <v>275</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
@@ -3733,10 +3745,10 @@
         <v>10</v>
       </c>
       <c r="B187" t="s">
-        <v>214</v>
+        <v>156</v>
       </c>
       <c r="C187" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
@@ -3744,7 +3756,7 @@
         <v>10</v>
       </c>
       <c r="B188" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C188" t="s">
         <v>216</v>
@@ -3755,10 +3767,10 @@
         <v>10</v>
       </c>
       <c r="B189" t="s">
-        <v>336</v>
+        <v>215</v>
       </c>
       <c r="C189" t="s">
-        <v>337</v>
+        <v>216</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
@@ -3766,10 +3778,10 @@
         <v>10</v>
       </c>
       <c r="B190" t="s">
-        <v>59</v>
+        <v>336</v>
       </c>
       <c r="C190" t="s">
-        <v>60</v>
+        <v>337</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
@@ -3777,10 +3789,10 @@
         <v>10</v>
       </c>
       <c r="B191" t="s">
-        <v>217</v>
+        <v>59</v>
       </c>
       <c r="C191" t="s">
-        <v>218</v>
+        <v>60</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
@@ -3788,10 +3800,10 @@
         <v>10</v>
       </c>
       <c r="B192" t="s">
-        <v>238</v>
+        <v>217</v>
       </c>
       <c r="C192" t="s">
-        <v>239</v>
+        <v>218</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
@@ -3799,10 +3811,10 @@
         <v>10</v>
       </c>
       <c r="B193" t="s">
-        <v>57</v>
+        <v>238</v>
       </c>
       <c r="C193" t="s">
-        <v>58</v>
+        <v>239</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
@@ -3810,10 +3822,10 @@
         <v>10</v>
       </c>
       <c r="B194" t="s">
-        <v>298</v>
+        <v>57</v>
       </c>
       <c r="C194" t="s">
-        <v>299</v>
+        <v>58</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
@@ -3821,10 +3833,10 @@
         <v>10</v>
       </c>
       <c r="B195" t="s">
-        <v>45</v>
+        <v>298</v>
       </c>
       <c r="C195" t="s">
-        <v>46</v>
+        <v>299</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
@@ -3832,10 +3844,10 @@
         <v>10</v>
       </c>
       <c r="B196" t="s">
-        <v>332</v>
+        <v>45</v>
       </c>
       <c r="C196" t="s">
-        <v>333</v>
+        <v>46</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
@@ -3843,10 +3855,10 @@
         <v>10</v>
       </c>
       <c r="B197" t="s">
-        <v>89</v>
+        <v>332</v>
       </c>
       <c r="C197" t="s">
-        <v>90</v>
+        <v>333</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
@@ -3854,10 +3866,10 @@
         <v>10</v>
       </c>
       <c r="B198" t="s">
-        <v>355</v>
+        <v>89</v>
       </c>
       <c r="C198" t="s">
-        <v>356</v>
+        <v>90</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
@@ -3865,10 +3877,10 @@
         <v>10</v>
       </c>
       <c r="B199" t="s">
-        <v>230</v>
+        <v>355</v>
       </c>
       <c r="C199" t="s">
-        <v>231</v>
+        <v>356</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
@@ -3876,10 +3888,10 @@
         <v>10</v>
       </c>
       <c r="B200" t="s">
-        <v>297</v>
+        <v>230</v>
       </c>
       <c r="C200" t="s">
-        <v>296</v>
+        <v>231</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
@@ -3887,7 +3899,7 @@
         <v>10</v>
       </c>
       <c r="B201" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C201" t="s">
         <v>296</v>
@@ -3898,10 +3910,10 @@
         <v>10</v>
       </c>
       <c r="B202" t="s">
-        <v>278</v>
+        <v>295</v>
       </c>
       <c r="C202" t="s">
-        <v>279</v>
+        <v>296</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
@@ -3909,10 +3921,10 @@
         <v>10</v>
       </c>
       <c r="B203" t="s">
-        <v>62</v>
+        <v>278</v>
       </c>
       <c r="C203" t="s">
-        <v>61</v>
+        <v>279</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
@@ -3920,10 +3932,10 @@
         <v>10</v>
       </c>
       <c r="B204" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="C204" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
@@ -3931,10 +3943,10 @@
         <v>10</v>
       </c>
       <c r="B205" t="s">
-        <v>135</v>
+        <v>47</v>
       </c>
       <c r="C205" t="s">
-        <v>136</v>
+        <v>48</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
@@ -3942,10 +3954,10 @@
         <v>10</v>
       </c>
       <c r="B206" t="s">
-        <v>366</v>
+        <v>135</v>
       </c>
       <c r="C206" t="s">
-        <v>367</v>
+        <v>136</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -3953,32 +3965,32 @@
         <v>10</v>
       </c>
       <c r="B207" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
       <c r="C207" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>10</v>
       </c>
-      <c r="B208" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="C208" s="1" t="s">
-        <v>192</v>
+      <c r="B208" t="s">
+        <v>351</v>
+      </c>
+      <c r="C208" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>10</v>
       </c>
-      <c r="B209" t="s">
-        <v>303</v>
-      </c>
-      <c r="C209" t="s">
-        <v>308</v>
+      <c r="B209" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C209" s="1" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
@@ -3986,10 +3998,10 @@
         <v>10</v>
       </c>
       <c r="B210" t="s">
-        <v>240</v>
+        <v>303</v>
       </c>
       <c r="C210" t="s">
-        <v>245</v>
+        <v>308</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
@@ -3997,10 +4009,10 @@
         <v>10</v>
       </c>
       <c r="B211" t="s">
-        <v>376</v>
+        <v>240</v>
       </c>
       <c r="C211" t="s">
-        <v>377</v>
+        <v>245</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
@@ -4008,10 +4020,10 @@
         <v>10</v>
       </c>
       <c r="B212" t="s">
-        <v>183</v>
+        <v>376</v>
       </c>
       <c r="C212" t="s">
-        <v>184</v>
+        <v>377</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
@@ -4019,10 +4031,10 @@
         <v>10</v>
       </c>
       <c r="B213" t="s">
-        <v>55</v>
+        <v>183</v>
       </c>
       <c r="C213" t="s">
-        <v>52</v>
+        <v>184</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
@@ -4030,10 +4042,10 @@
         <v>10</v>
       </c>
       <c r="B214" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="C214" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
@@ -4041,10 +4053,10 @@
         <v>10</v>
       </c>
       <c r="B215" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C215" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
@@ -4052,10 +4064,10 @@
         <v>10</v>
       </c>
       <c r="B216" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C216" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
@@ -4063,10 +4075,10 @@
         <v>10</v>
       </c>
       <c r="B217" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C217" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
@@ -4074,10 +4086,10 @@
         <v>10</v>
       </c>
       <c r="B218" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="C218" t="s">
-        <v>61</v>
+        <v>27</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
@@ -4085,10 +4097,10 @@
         <v>10</v>
       </c>
       <c r="B219" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C219" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
@@ -4096,10 +4108,10 @@
         <v>10</v>
       </c>
       <c r="B220" t="s">
-        <v>405</v>
+        <v>15</v>
       </c>
       <c r="C220" t="s">
-        <v>406</v>
+        <v>14</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
@@ -4107,10 +4119,10 @@
         <v>10</v>
       </c>
       <c r="B221" t="s">
-        <v>340</v>
+        <v>405</v>
       </c>
       <c r="C221" t="s">
-        <v>341</v>
+        <v>406</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
@@ -4118,10 +4130,10 @@
         <v>10</v>
       </c>
       <c r="B222" t="s">
-        <v>85</v>
+        <v>340</v>
       </c>
       <c r="C222" t="s">
-        <v>86</v>
+        <v>341</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
@@ -4129,10 +4141,10 @@
         <v>10</v>
       </c>
       <c r="B223" t="s">
-        <v>418</v>
+        <v>85</v>
       </c>
       <c r="C223" t="s">
-        <v>419</v>
+        <v>86</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
@@ -4140,10 +4152,10 @@
         <v>10</v>
       </c>
       <c r="B224" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C224" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
@@ -4151,16 +4163,49 @@
         <v>10</v>
       </c>
       <c r="B225" t="s">
+        <v>420</v>
+      </c>
+      <c r="C225" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>10</v>
+      </c>
+      <c r="B226" t="s">
         <v>422</v>
       </c>
-      <c r="C225" t="s">
+      <c r="C226" t="s">
         <v>423</v>
       </c>
     </row>
+    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>10</v>
+      </c>
+      <c r="B227" t="s">
+        <v>425</v>
+      </c>
+      <c r="C227" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>10</v>
+      </c>
+      <c r="B228" t="s">
+        <v>427</v>
+      </c>
+      <c r="C228" t="s">
+        <v>426</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C222">
-    <sortCondition ref="A2:A222"/>
-    <sortCondition ref="B2:B222"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C223">
+    <sortCondition ref="A2:A223"/>
+    <sortCondition ref="B2:B223"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>